<commit_message>
Operational Constraints + Discussion on allocation model validation by (Cadorel and Saingre 2024)
</commit_message>
<xml_diff>
--- a/literature-management.xlsx
+++ b/literature-management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jay/phd/papers/sok - a survey on software power monitoring tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{E1594412-51E6-4844-98FA-0862AD025FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{20DCD17C-6B36-A94F-BDAE-891B995E3F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="920" windowWidth="30080" windowHeight="18580" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1002,9 +1002,6 @@
     <t>Delegated to another tool</t>
   </si>
   <si>
-    <t>( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</t>
-  </si>
-  <si>
     <t>Network (NIC)</t>
   </si>
   <si>
@@ -1200,10 +1197,6 @@
 proportionnaly to processes size</t>
   </si>
   <si>
-    <t>✗(available for estimations in virtualised
-context )</t>
-  </si>
-  <si>
     <t>Linux</t>
   </si>
   <si>
@@ -1242,14 +1235,6 @@
     <t>Regression model (# CPU and OS-provided Resource Utilisation metrics as input)</t>
   </si>
   <si>
-    <t xml:space="preserve">XGBoost Model (#CPU TDP, CPU Frequency and CPU % as input)
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✗XGBoost model for system-level estimations in virtualised
-contex (TDP) </t>
-  </si>
-  <si>
     <t>✗Regression-based models for VM deployment</t>
   </si>
   <si>
@@ -1258,10 +1243,6 @@
   </si>
   <si>
     <t>✗HPC vector (cycles, instructions, cache misses)</t>
-  </si>
-  <si>
-    <t>✗XGBoost (TDP)
-or Regression-based (TDP)</t>
   </si>
   <si>
     <t>OS-provided PID CPU %
@@ -1302,6 +1283,25 @@
     <t>Modeled and 
 allocated to container 
 according to OS-provided PID CPU %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✗1) XGBoost model (TDP, Machine Specs and CPU%)
+2) Analytical Model(TDP, #CPUchips and CPU %) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1) XGBoost model (TDP, Machine Specs and CPU%)
+2) Analytical Model(TDP, #CPUchips and CPU %) </t>
+  </si>
+  <si>
+    <t>Regression-based model</t>
+  </si>
+  <si>
+    <t>no
+( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</t>
+  </si>
+  <si>
+    <t>OS-provided PID CPU %
+Cgroups Stat</t>
   </si>
 </sst>
 </file>
@@ -1683,7 +1683,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -2416,30 +2416,97 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="44" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="129">
+  <dxfs count="121">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3217,33 +3284,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -3410,126 +3450,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3745,13 +3665,13 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{DF00C389-F294-FB48-80B0-022781D38C47}">
-      <tableStyleElement type="wholeTable" dxfId="128"/>
+      <tableStyleElement type="wholeTable" dxfId="120"/>
     </tableStyle>
     <tableStyle name="Table Style 2" pivot="0" count="4" xr9:uid="{66177898-DED3-9C47-8DA6-ABD521A19111}">
-      <tableStyleElement type="wholeTable" dxfId="127"/>
-      <tableStyleElement type="headerRow" dxfId="126"/>
-      <tableStyleElement type="firstRowStripe" dxfId="125"/>
-      <tableStyleElement type="secondRowStripe" dxfId="124"/>
+      <tableStyleElement type="wholeTable" dxfId="119"/>
+      <tableStyleElement type="headerRow" dxfId="118"/>
+      <tableStyleElement type="firstRowStripe" dxfId="117"/>
+      <tableStyleElement type="secondRowStripe" dxfId="116"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -3766,18 +3686,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C9355DD-35BE-3D46-8331-B67246AE3C74}" name="Table1" displayName="Table1" ref="C2:K22" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122" tableBorderDxfId="121">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C9355DD-35BE-3D46-8331-B67246AE3C74}" name="Table1" displayName="Table1" ref="C2:K22" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114" tableBorderDxfId="113">
   <autoFilter ref="C2:K22" xr:uid="{1C9355DD-35BE-3D46-8331-B67246AE3C74}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B697189A-DF2B-4341-9FF4-7259FA9252F8}" name="Tool Name" dataDxfId="120"/>
-    <tableColumn id="2" xr3:uid="{F3B719A6-5185-6144-A373-7DD05C5FE758}" name="References" dataDxfId="119"/>
-    <tableColumn id="3" xr3:uid="{271ED028-8F14-D741-A569-E2FEB926BB1C}" name="Year" dataDxfId="118"/>
-    <tableColumn id="4" xr3:uid="{B7FF3EF8-B658-904B-8045-D98673D5126F}" name="Authors/Institution" dataDxfId="117"/>
-    <tableColumn id="5" xr3:uid="{63D16556-412F-8B4C-BF7C-5FF77216838E}" name="Discovery Method" dataDxfId="116"/>
-    <tableColumn id="6" xr3:uid="{946E4FD2-8FE0-9345-A39D-83A4386577DF}" name="Discovered From" dataDxfId="115"/>
-    <tableColumn id="7" xr3:uid="{DF93B5C3-BD8E-D543-8F4C-AC0C5199BC07}" name="Selection Status" dataDxfId="114"/>
-    <tableColumn id="8" xr3:uid="{03969A93-C0C5-BB4C-ACA8-090EAA97265A}" name="Exclusion Reason" dataDxfId="113"/>
-    <tableColumn id="9" xr3:uid="{01558EB7-81C3-6642-A7E2-29E574F37760}" name="Short Description" dataDxfId="112"/>
+    <tableColumn id="1" xr3:uid="{B697189A-DF2B-4341-9FF4-7259FA9252F8}" name="Tool Name" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{F3B719A6-5185-6144-A373-7DD05C5FE758}" name="References" dataDxfId="111"/>
+    <tableColumn id="3" xr3:uid="{271ED028-8F14-D741-A569-E2FEB926BB1C}" name="Year" dataDxfId="110"/>
+    <tableColumn id="4" xr3:uid="{B7FF3EF8-B658-904B-8045-D98673D5126F}" name="Authors/Institution" dataDxfId="109"/>
+    <tableColumn id="5" xr3:uid="{63D16556-412F-8B4C-BF7C-5FF77216838E}" name="Discovery Method" dataDxfId="108"/>
+    <tableColumn id="6" xr3:uid="{946E4FD2-8FE0-9345-A39D-83A4386577DF}" name="Discovered From" dataDxfId="107"/>
+    <tableColumn id="7" xr3:uid="{DF93B5C3-BD8E-D543-8F4C-AC0C5199BC07}" name="Selection Status" dataDxfId="106"/>
+    <tableColumn id="8" xr3:uid="{03969A93-C0C5-BB4C-ACA8-090EAA97265A}" name="Exclusion Reason" dataDxfId="105"/>
+    <tableColumn id="9" xr3:uid="{01558EB7-81C3-6642-A7E2-29E574F37760}" name="Short Description" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4450,13 +4370,13 @@
         <v>44</v>
       </c>
       <c r="D14" s="46" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E14" s="10">
         <v>2014</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G14" s="17" t="s">
         <v>98</v>
@@ -4471,7 +4391,7 @@
         <v>35</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="2:11" ht="16">
@@ -4499,7 +4419,7 @@
     <row r="16" spans="2:11">
       <c r="B16" s="10"/>
       <c r="C16" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D16" s="46"/>
       <c r="E16" s="10"/>
@@ -5003,10 +4923,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="I3:I16">
-    <cfRule type="beginsWith" dxfId="99" priority="1" operator="beginsWith" text="Not">
+    <cfRule type="beginsWith" dxfId="103" priority="1" operator="beginsWith" text="Not">
       <formula>LEFT(I3,LEN("Not"))="Not"</formula>
     </cfRule>
-    <cfRule type="beginsWith" dxfId="98" priority="2" operator="beginsWith" text="Selected">
+    <cfRule type="beginsWith" dxfId="102" priority="2" operator="beginsWith" text="Selected">
       <formula>LEFT(I3,LEN("Selected"))="Selected"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5300,7 +5220,7 @@
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="30" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>55</v>
@@ -7721,7 +7641,7 @@
       <c r="AI2" s="78"/>
       <c r="AJ2"/>
       <c r="AK2" s="91" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AL2" s="91"/>
       <c r="AM2" s="91"/>
@@ -7768,7 +7688,7 @@
     <row r="3" spans="1:163" ht="47" customHeight="1">
       <c r="B3" s="87"/>
       <c r="D3" s="72" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E3" s="88" t="s">
         <v>261</v>
@@ -7777,7 +7697,7 @@
         <v>262</v>
       </c>
       <c r="G3" s="88" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H3" s="88" t="s">
         <v>263</v>
@@ -7810,7 +7730,7 @@
       <c r="Y3" s="83"/>
       <c r="Z3" s="64"/>
       <c r="AA3" s="81" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AB3" s="82"/>
       <c r="AC3" s="82"/>
@@ -7824,19 +7744,19 @@
       <c r="AI3" s="83"/>
       <c r="AJ3" s="64"/>
       <c r="AK3" s="84" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AL3" s="84"/>
       <c r="AM3" s="84"/>
       <c r="AN3" s="84"/>
       <c r="AO3" s="85" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AQ3" s="86" t="s">
         <v>279</v>
       </c>
       <c r="AR3" s="86" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AS3" s="86" t="s">
         <v>280</v>
@@ -7857,7 +7777,7 @@
         <v>274</v>
       </c>
       <c r="AZ3" s="76" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BA3" s="76"/>
       <c r="BB3" s="76"/>
@@ -7890,7 +7810,7 @@
         <v>82</v>
       </c>
       <c r="BT3" s="79" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="BU3" s="79"/>
       <c r="BV3" s="79"/>
@@ -7905,61 +7825,61 @@
       <c r="I4" s="88"/>
       <c r="J4" s="88"/>
       <c r="L4" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="M4" s="89"/>
       <c r="N4" s="89"/>
       <c r="O4" s="89" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P4" s="64"/>
       <c r="Q4" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="R4" s="89"/>
       <c r="S4" s="89"/>
       <c r="T4" s="89" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="U4" s="64"/>
       <c r="V4" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="W4" s="89"/>
       <c r="X4" s="89"/>
       <c r="Y4" s="89" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Z4" s="64"/>
       <c r="AA4" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AB4" s="89"/>
       <c r="AC4" s="89"/>
       <c r="AD4" s="89" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AE4" s="64"/>
       <c r="AF4" s="89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AG4" s="89"/>
       <c r="AH4" s="89"/>
       <c r="AI4" s="89" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AJ4" s="64"/>
       <c r="AK4" s="84" t="s">
+        <v>322</v>
+      </c>
+      <c r="AL4" s="140" t="s">
         <v>323</v>
-      </c>
-      <c r="AL4" s="140" t="s">
-        <v>324</v>
       </c>
       <c r="AM4" s="84" t="s">
         <v>268</v>
       </c>
       <c r="AN4" s="84" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AO4" s="85"/>
       <c r="AQ4" s="86"/>
@@ -7977,7 +7897,7 @@
         <v>68</v>
       </c>
       <c r="BB4" s="76" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="BC4" s="76" t="s">
         <v>66</v>
@@ -7986,10 +7906,10 @@
         <v>62</v>
       </c>
       <c r="BE4" s="76" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BF4" s="142" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="BG4" s="143"/>
       <c r="BH4" s="144"/>
@@ -8003,7 +7923,7 @@
         <v>76</v>
       </c>
       <c r="BL4" s="67" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="BN4" s="79"/>
       <c r="BO4" s="79"/>
@@ -8106,13 +8026,13 @@
       <c r="BD5" s="76"/>
       <c r="BE5" s="76"/>
       <c r="BF5" s="63" t="s">
+        <v>343</v>
+      </c>
+      <c r="BG5" s="63" t="s">
+        <v>344</v>
+      </c>
+      <c r="BH5" s="63" t="s">
         <v>345</v>
-      </c>
-      <c r="BG5" s="63" t="s">
-        <v>346</v>
-      </c>
-      <c r="BH5" s="63" t="s">
-        <v>347</v>
       </c>
       <c r="BI5" s="76"/>
       <c r="BJ5" s="76"/>
@@ -8215,11 +8135,11 @@
       <c r="AG7" s="58" t="s">
         <v>132</v>
       </c>
-      <c r="AH7" s="56" t="s">
-        <v>344</v>
+      <c r="AH7" s="58" t="s">
+        <v>107</v>
       </c>
       <c r="AI7" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AJ7" s="64"/>
       <c r="AK7" s="58" t="s">
@@ -8314,7 +8234,7 @@
     </row>
     <row r="8" spans="1:163" s="59" customFormat="1" ht="409.6">
       <c r="B8" s="61" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C8"/>
       <c r="D8" s="56" t="s">
@@ -8345,10 +8265,10 @@
         <v>111</v>
       </c>
       <c r="N8" s="56" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="O8" s="56" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="P8" s="64"/>
       <c r="Q8" s="56" t="s">
@@ -8361,7 +8281,7 @@
         <v>107</v>
       </c>
       <c r="T8" s="56" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="U8" s="64"/>
       <c r="V8" s="56" t="s">
@@ -8374,7 +8294,7 @@
         <v>107</v>
       </c>
       <c r="Y8" s="56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="Z8" s="64"/>
       <c r="AA8" s="58" t="s">
@@ -8391,16 +8311,16 @@
       </c>
       <c r="AE8" s="64"/>
       <c r="AF8" s="58" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="AG8" s="58" t="s">
         <v>107</v>
       </c>
       <c r="AH8" s="58" t="s">
-        <v>290</v>
+        <v>369</v>
       </c>
       <c r="AI8" s="56" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="AJ8" s="64"/>
       <c r="AK8" s="58" t="s">
@@ -8416,13 +8336,13 @@
         <v>107</v>
       </c>
       <c r="AO8" s="58" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="AQ8" s="56" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AR8" s="56" t="s">
-        <v>281</v>
+        <v>370</v>
       </c>
       <c r="AS8" s="58" t="s">
         <v>107</v>
@@ -8509,7 +8429,7 @@
     </row>
     <row r="9" spans="1:163" s="59" customFormat="1" ht="409.6">
       <c r="B9" s="61" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C9"/>
       <c r="D9" s="56" t="s">
@@ -8540,10 +8460,10 @@
         <v>111</v>
       </c>
       <c r="N9" s="56" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="O9" s="56" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="P9" s="64"/>
       <c r="Q9" s="56" t="s">
@@ -8556,7 +8476,7 @@
         <v>107</v>
       </c>
       <c r="T9" s="56" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="U9" s="64"/>
       <c r="V9" s="56" t="s">
@@ -8569,7 +8489,7 @@
         <v>107</v>
       </c>
       <c r="Y9" s="56" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="Z9" s="64"/>
       <c r="AA9" s="58" t="s">
@@ -8586,38 +8506,38 @@
       </c>
       <c r="AE9" s="64"/>
       <c r="AF9" s="58" t="s">
+        <v>288</v>
+      </c>
+      <c r="AG9" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="AH9" s="58" t="s">
         <v>289</v>
       </c>
-      <c r="AG9" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="AH9" s="58" t="s">
-        <v>290</v>
-      </c>
       <c r="AI9" s="56" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="AJ9" s="64"/>
       <c r="AK9" s="58" t="s">
         <v>107</v>
       </c>
       <c r="AL9" s="58" t="s">
+        <v>341</v>
+      </c>
+      <c r="AM9" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="AN9" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="AO9" s="58" t="s">
         <v>342</v>
       </c>
-      <c r="AM9" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="AN9" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="AO9" s="58" t="s">
-        <v>343</v>
-      </c>
       <c r="AQ9" s="56" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="AR9" s="56" t="s">
-        <v>281</v>
+        <v>370</v>
       </c>
       <c r="AS9" s="58" t="s">
         <v>107</v>
@@ -8626,7 +8546,7 @@
         <v>141</v>
       </c>
       <c r="AV9" s="58" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="AW9" s="58"/>
       <c r="AX9" s="58" t="s">
@@ -8730,16 +8650,16 @@
         <v>273</v>
       </c>
       <c r="L10" s="56" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M10" s="58" t="s">
         <v>132</v>
       </c>
       <c r="N10" s="56" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="O10" s="56" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="P10" s="64"/>
       <c r="Q10" s="56" t="s">
@@ -8752,7 +8672,7 @@
         <v>107</v>
       </c>
       <c r="T10" s="56" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="U10" s="64"/>
       <c r="V10" s="56" t="s">
@@ -8765,7 +8685,7 @@
         <v>107</v>
       </c>
       <c r="Y10" s="56" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="Z10" s="64"/>
       <c r="AA10" s="58" t="s">
@@ -8785,13 +8705,13 @@
         <v>60</v>
       </c>
       <c r="AG10" s="58" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="AH10" s="56" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="AI10" s="58" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="AJ10" s="64"/>
       <c r="AK10" s="60" t="s">
@@ -8807,10 +8727,10 @@
         <v>273</v>
       </c>
       <c r="AO10" s="58" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="AQ10" s="56" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="AR10" s="58" t="s">
         <v>107</v>
@@ -8828,10 +8748,10 @@
         <v>148</v>
       </c>
       <c r="AX10" s="58" t="s">
+        <v>301</v>
+      </c>
+      <c r="AY10" s="58" t="s">
         <v>302</v>
-      </c>
-      <c r="AY10" s="58" t="s">
-        <v>303</v>
       </c>
       <c r="AZ10" s="58" t="s">
         <v>122</v>
@@ -8936,10 +8856,10 @@
         <v>107</v>
       </c>
       <c r="N12" s="56" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O12" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="P12" s="64"/>
       <c r="Q12" s="58" t="s">
@@ -8978,7 +8898,7 @@
         <v>60</v>
       </c>
       <c r="AD12" s="56" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AE12" s="64"/>
       <c r="AF12" s="58" t="s">
@@ -8988,10 +8908,10 @@
         <v>107</v>
       </c>
       <c r="AH12" s="56" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AI12" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AJ12" s="64"/>
       <c r="AK12" s="58" t="s">
@@ -9119,10 +9039,10 @@
         <v>107</v>
       </c>
       <c r="N13" s="56" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="O13" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="P13" s="64"/>
       <c r="Q13" s="58" t="s">
@@ -9171,10 +9091,10 @@
         <v>107</v>
       </c>
       <c r="AH13" s="56" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="AI13" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AJ13" s="64"/>
       <c r="AK13" s="58" t="s">
@@ -9304,7 +9224,7 @@
         <v>107</v>
       </c>
       <c r="O14" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="P14" s="64"/>
       <c r="Q14" s="58" t="s">
@@ -9317,20 +9237,20 @@
         <v>107</v>
       </c>
       <c r="T14" s="56" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="U14" s="64"/>
       <c r="V14" s="58" t="s">
         <v>107</v>
       </c>
       <c r="W14" s="58" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="X14" s="58" t="s">
         <v>107</v>
       </c>
       <c r="Y14" s="56" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="Z14" s="64"/>
       <c r="AA14" s="58" t="s">
@@ -9356,7 +9276,7 @@
         <v>245</v>
       </c>
       <c r="AI14" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AJ14" s="64"/>
       <c r="AK14" s="58" t="s">
@@ -9396,7 +9316,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="58" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AZ14" s="58" t="s">
         <v>60</v>
@@ -9502,7 +9422,7 @@
         <v>107</v>
       </c>
       <c r="O15" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="P15" s="64"/>
       <c r="Q15" s="58" t="s">
@@ -9515,20 +9435,20 @@
         <v>107</v>
       </c>
       <c r="T15" s="56" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="U15" s="64"/>
       <c r="V15" s="58" t="s">
         <v>107</v>
       </c>
       <c r="W15" s="58" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="X15" s="58" t="s">
         <v>107</v>
       </c>
       <c r="Y15" s="56" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="Z15" s="64"/>
       <c r="AA15" s="58" t="s">
@@ -9554,7 +9474,7 @@
         <v>245</v>
       </c>
       <c r="AI15" s="56" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AJ15" s="64"/>
       <c r="AK15" s="58" t="s">
@@ -9570,7 +9490,7 @@
         <v>107</v>
       </c>
       <c r="AO15" s="58" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="AQ15" s="58" t="s">
         <v>107</v>
@@ -9588,7 +9508,7 @@
         <v>229</v>
       </c>
       <c r="AW15" s="58" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AX15" s="58" t="s">
         <v>107</v>
@@ -9701,10 +9621,10 @@
         <v>107</v>
       </c>
       <c r="N17" s="56" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="O17" s="56" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="P17" s="64"/>
       <c r="Q17" s="58" t="s">
@@ -9740,10 +9660,10 @@
         <v>107</v>
       </c>
       <c r="AC17" s="58" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AD17" s="56" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AE17" s="64"/>
       <c r="AF17" s="58" t="s">
@@ -9760,16 +9680,16 @@
       </c>
       <c r="AJ17" s="64"/>
       <c r="AK17" s="58" t="s">
+        <v>305</v>
+      </c>
+      <c r="AL17" s="62" t="s">
+        <v>107</v>
+      </c>
+      <c r="AM17" s="58" t="s">
         <v>306</v>
       </c>
-      <c r="AL17" s="62" t="s">
-        <v>107</v>
-      </c>
-      <c r="AM17" s="58" t="s">
+      <c r="AN17" s="58" t="s">
         <v>307</v>
-      </c>
-      <c r="AN17" s="58" t="s">
-        <v>308</v>
       </c>
       <c r="AO17" s="58" t="s">
         <v>107</v>
@@ -9825,7 +9745,7 @@
         <v>107</v>
       </c>
       <c r="BL17" s="58" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="BN17" s="56"/>
       <c r="BO17" s="56" t="s">
@@ -9875,39 +9795,39 @@
         <v>107</v>
       </c>
       <c r="M18" s="56" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="N18" s="56" t="s">
         <v>107</v>
       </c>
       <c r="O18" s="56" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="P18" s="64"/>
       <c r="Q18" s="58" t="s">
         <v>107</v>
       </c>
       <c r="R18" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="S18" s="56" t="s">
         <v>107</v>
       </c>
       <c r="T18" s="56" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="U18" s="64"/>
       <c r="V18" s="58" t="s">
         <v>107</v>
       </c>
       <c r="W18" s="58" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="X18" s="58" t="s">
         <v>107</v>
       </c>
       <c r="Y18" s="56" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="Z18" s="64"/>
       <c r="AA18" s="58" t="s">
@@ -9933,7 +9853,7 @@
         <v>245</v>
       </c>
       <c r="AI18" s="56" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="AJ18" s="64"/>
       <c r="AK18" s="58" t="s">
@@ -10006,7 +9926,7 @@
         <v>107</v>
       </c>
       <c r="BL18" s="58" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="BN18" s="56" t="s">
         <v>214</v>
@@ -10022,7 +9942,7 @@
       </c>
       <c r="BR18" s="56"/>
       <c r="BS18" s="56" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="BT18" s="58" t="s">
         <v>107</v>
@@ -10070,7 +9990,7 @@
         <v>107</v>
       </c>
       <c r="O19" s="56" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="P19" s="64"/>
       <c r="Q19" s="58" t="s">
@@ -10160,7 +10080,7 @@
         <v>107</v>
       </c>
       <c r="AY19" s="58" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="AZ19" s="58" t="s">
         <v>60</v>
@@ -10251,26 +10171,26 @@
         <v>107</v>
       </c>
       <c r="M20" s="56" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="N20" s="56" t="s">
         <v>107</v>
       </c>
       <c r="O20" s="56" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="P20" s="64"/>
       <c r="Q20" s="58" t="s">
         <v>107</v>
       </c>
       <c r="R20" s="56" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="S20" s="58" t="s">
         <v>107</v>
       </c>
       <c r="T20" s="56" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="U20" s="64"/>
       <c r="V20" s="58" t="s">
@@ -10303,13 +10223,13 @@
         <v>107</v>
       </c>
       <c r="AG20" s="56" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AH20" s="58" t="s">
         <v>107</v>
       </c>
       <c r="AI20" s="56" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AJ20" s="64"/>
       <c r="AK20" s="58" t="s">
@@ -10340,73 +10260,73 @@
         <v>107</v>
       </c>
       <c r="AV20" s="58" t="s">
+        <v>333</v>
+      </c>
+      <c r="AW20" s="58" t="s">
+        <v>338</v>
+      </c>
+      <c r="AX20" s="58" t="s">
+        <v>335</v>
+      </c>
+      <c r="AY20" s="58" t="s">
         <v>334</v>
       </c>
-      <c r="AW20" s="58" t="s">
-        <v>339</v>
-      </c>
-      <c r="AX20" s="58" t="s">
+      <c r="AZ20" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="BA20" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="BB20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BC20" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="BD20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BE20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BF20" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="BG20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BH20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BI20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BJ20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BK20" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="BL20" s="58" t="s">
+        <v>311</v>
+      </c>
+      <c r="BN20" s="56" t="s">
         <v>336</v>
-      </c>
-      <c r="AY20" s="58" t="s">
-        <v>335</v>
-      </c>
-      <c r="AZ20" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="BA20" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="BB20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BC20" s="58" t="s">
-        <v>60</v>
-      </c>
-      <c r="BD20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BE20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BF20" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="BG20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BH20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BI20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BJ20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BK20" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="BL20" s="58" t="s">
-        <v>312</v>
-      </c>
-      <c r="BN20" s="56" t="s">
-        <v>337</v>
       </c>
       <c r="BO20" s="56" t="s">
         <v>120</v>
       </c>
       <c r="BP20" s="56" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="BQ20" s="56" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="BR20" s="56" t="s">
         <v>178</v>
       </c>
       <c r="BS20" s="56" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="BT20" s="58" t="s">
         <v>107</v>
@@ -10556,423 +10476,439 @@
     <mergeCell ref="AF3:AI3"/>
   </mergeCells>
   <conditionalFormatting sqref="V12:X12 Y14:Y15 D14:J15 D12:J12 L12:O12 D7:J10 AA7:AD10 BN7:BV10 AU17:AU20 D17:J20 AK12:AO12 AK14:AO15 AK17:AO20 BN12:BV15 BN17:BV20 AK7:AO10 L14:N15">
-    <cfRule type="endsWith" dxfId="97" priority="296" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="101" priority="300" operator="endsWith" text="no">
       <formula>RIGHT(D7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14:J15 D12:J12 L12:O12 Y14:Y15 V12:Y12 D7:J10 AA7:AD10 BN7:BV10 AU17:AU20 D17:J20 AK12:AO12 AK14:AO15 AK17:AO20 BN12:BV15 BN17:BV20 AK7:AO10 L14:N15">
-    <cfRule type="expression" dxfId="96" priority="295">
+    <cfRule type="expression" dxfId="100" priority="299">
       <formula>TRIM(LOWER(D7))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q14:T15 Q12:T12 AA14:AD15 AA12:AD12 AQ14:AS15 AQ12:AS12 AV12:BL12 AF12:AI12 L7:O10 L17:O20 Q17:T20 V17:Y20 AA17:AD20 AF17:AI20 AQ17:AS20 AV17:BL20 AV14:BL15 AF14:AI15 AF13:AG13 AI13">
-    <cfRule type="expression" dxfId="95" priority="217">
+    <cfRule type="expression" dxfId="99" priority="221">
       <formula>TRIM(LOWER(L7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="94" priority="218" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="98" priority="222" operator="endsWith" text="no">
       <formula>RIGHT(L7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q7:T10">
-    <cfRule type="expression" dxfId="93" priority="155">
+    <cfRule type="expression" dxfId="97" priority="159">
       <formula>TRIM(LOWER(Q7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="92" priority="156" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="96" priority="160" operator="endsWith" text="no">
       <formula>RIGHT(Q7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R17">
-    <cfRule type="expression" dxfId="91" priority="199">
+    <cfRule type="expression" dxfId="95" priority="203">
       <formula>TRIM(LOWER(R17))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="90" priority="200" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="94" priority="204" operator="endsWith" text="no">
       <formula>RIGHT(R17,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V15:X15">
-    <cfRule type="expression" dxfId="89" priority="131">
+    <cfRule type="expression" dxfId="93" priority="135">
       <formula>TRIM(LOWER(V15))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="88" priority="132" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="92" priority="136" operator="endsWith" text="no">
       <formula>RIGHT(V15,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V7:Y10">
-    <cfRule type="expression" dxfId="87" priority="157">
+    <cfRule type="expression" dxfId="91" priority="161">
       <formula>TRIM(LOWER(V7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="86" priority="158" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="90" priority="162" operator="endsWith" text="no">
       <formula>RIGHT(V7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V14:Y14">
-    <cfRule type="expression" dxfId="85" priority="167">
+    <cfRule type="expression" dxfId="89" priority="171">
       <formula>TRIM(LOWER(V14))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="84" priority="170" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="88" priority="174" operator="endsWith" text="no">
       <formula>RIGHT(V14,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y12:Y13">
-    <cfRule type="endsWith" dxfId="83" priority="124" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="87" priority="128" operator="endsWith" text="no">
       <formula>RIGHT(Y12,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF7:AI10">
-    <cfRule type="expression" dxfId="82" priority="95">
+    <cfRule type="expression" dxfId="86" priority="99">
       <formula>TRIM(LOWER(AF7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="81" priority="96" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="85" priority="100" operator="endsWith" text="no">
       <formula>RIGHT(AF7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ14:AS15 AQ12:AS12 D14:J15 D12:J12 L12:O12 Q14:T15 Q12:T12 V14:Y15 V12:Y12 AA14:AD15 AA12:AD12 AF12:AI12 D7:J10 V7:Y10 AA7:AD10 BN7:BV10 D17:J20 L17:O20 Q17:T20 V17:Y20 AA17:AD20 AF17:AI20 AK12:AO12 AK14:AO15 AK17:AO20 AQ17:AS20 BN12:BV15 BN17:BV20 AK7:AO10 AQ7:AS10 L7:O10 L14:N15 AU7:BL10 AU12:BL12 AU17:BL20 AU14:BL15 AF14:AI15 AF13:AG13 AI13 Q7:T10 AF7:AI10">
-    <cfRule type="containsBlanks" dxfId="80" priority="47">
+  <conditionalFormatting sqref="AQ14:AS15 AQ12:AS12 D14:J15 D12:J12 L12:O12 Q14:T15 Q12:T12 V14:Y15 V12:Y12 AA14:AD15 AA12:AD12 AF12:AI12 D7:J10 V7:Y10 AA7:AD10 BN7:BV10 D17:J20 L17:O20 Q17:T20 V17:Y20 AA17:AD20 AF17:AI20 AK12:AO12 AK14:AO15 AK17:AO20 AQ17:AS20 BN12:BV15 BN17:BV20 AK7:AO10 L14:N15 AU7:BL10 AU12:BL12 AU17:BL20 AU14:BL15 AF14:AI15 AF13:AG13 AI13 Q7:T10 L7:O10 AQ7:AS10 AF7:AI10">
+    <cfRule type="containsBlanks" dxfId="2" priority="51">
       <formula>LEN(TRIM(D7))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AQ7:AS10">
-    <cfRule type="expression" dxfId="79" priority="97">
+    <cfRule type="expression" dxfId="1" priority="101">
       <formula>TRIM(LOWER(AQ7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="78" priority="98" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="0" priority="102" operator="endsWith" text="no">
       <formula>RIGHT(AQ7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR7">
-    <cfRule type="expression" dxfId="77" priority="83">
+    <cfRule type="expression" dxfId="84" priority="87">
       <formula>TRIM(LOWER(AR7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="76" priority="84" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="83" priority="88" operator="endsWith" text="no">
       <formula>RIGHT(AR7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR14">
-    <cfRule type="expression" dxfId="75" priority="81">
+    <cfRule type="expression" dxfId="82" priority="85">
       <formula>TRIM(LOWER(AR14))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="74" priority="82" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="81" priority="86" operator="endsWith" text="no">
       <formula>RIGHT(AR14,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AV7:BL10">
-    <cfRule type="expression" dxfId="73" priority="93">
+    <cfRule type="expression" dxfId="80" priority="97">
       <formula>TRIM(LOWER(AV7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="72" priority="94" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="79" priority="98" operator="endsWith" text="no">
       <formula>RIGHT(AV7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY8:AY10">
-    <cfRule type="expression" dxfId="71" priority="89">
+    <cfRule type="expression" dxfId="78" priority="93">
       <formula>TRIM(LOWER(AY8))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="70" priority="90" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="77" priority="94" operator="endsWith" text="no">
       <formula>RIGHT(AY8,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V13:X13 D13:J13 L13:O13 AK13 AM13:AO13">
-    <cfRule type="endsWith" dxfId="69" priority="80" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="76" priority="84" operator="endsWith" text="no">
       <formula>RIGHT(D13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13:J13 L13:O13 AK13 V13:Y13 AM13:AO13">
-    <cfRule type="expression" dxfId="68" priority="79">
+    <cfRule type="expression" dxfId="75" priority="83">
       <formula>TRIM(LOWER(D13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q13:T13 AA13:AB13 AQ13:AS13 AU13:BE13 BI13:BL13">
-    <cfRule type="expression" dxfId="67" priority="77">
+    <cfRule type="expression" dxfId="74" priority="81">
       <formula>TRIM(LOWER(Q13))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="66" priority="78" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="73" priority="82" operator="endsWith" text="no">
       <formula>RIGHT(Q13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AQ13:AS13 D13:J13 L13:O13 Q13:T13 V13:Y13 AA13:AB13 AK13 AM13:AO13 AU13:BE13 BI13:BL13">
-    <cfRule type="containsBlanks" dxfId="65" priority="72">
+    <cfRule type="containsBlanks" dxfId="72" priority="76">
       <formula>LEN(TRIM(D13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU14:AU15 AU12 AU8:AU10">
-    <cfRule type="endsWith" dxfId="64" priority="76" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="71" priority="80" operator="endsWith" text="no">
       <formula>RIGHT(AU8,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU14:AU15 AU12 AU8:AU10">
-    <cfRule type="expression" dxfId="63" priority="75">
+    <cfRule type="expression" dxfId="70" priority="79">
       <formula>TRIM(LOWER(AU8))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU13">
-    <cfRule type="endsWith" dxfId="62" priority="74" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="69" priority="78" operator="endsWith" text="no">
       <formula>RIGHT(AU13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU13">
-    <cfRule type="expression" dxfId="61" priority="73">
+    <cfRule type="expression" dxfId="68" priority="77">
       <formula>TRIM(LOWER(AU13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L20">
-    <cfRule type="endsWith" dxfId="60" priority="71" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="67" priority="75" operator="endsWith" text="no">
       <formula>RIGHT(L20,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L20">
-    <cfRule type="expression" dxfId="59" priority="70">
+    <cfRule type="expression" dxfId="66" priority="74">
       <formula>TRIM(LOWER(L20))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL13">
-    <cfRule type="endsWith" dxfId="58" priority="69" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="65" priority="73" operator="endsWith" text="no">
       <formula>RIGHT(AL13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL13">
-    <cfRule type="expression" dxfId="57" priority="68">
+    <cfRule type="expression" dxfId="64" priority="72">
       <formula>TRIM(LOWER(AL13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL13">
-    <cfRule type="containsBlanks" dxfId="56" priority="67">
+    <cfRule type="containsBlanks" dxfId="63" priority="71">
       <formula>LEN(TRIM(AL13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU7">
-    <cfRule type="expression" dxfId="55" priority="53">
+    <cfRule type="expression" dxfId="62" priority="57">
       <formula>TRIM(LOWER(AU7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="54" priority="54" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="61" priority="58" operator="endsWith" text="no">
       <formula>RIGHT(AU7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU20">
-    <cfRule type="expression" dxfId="53" priority="51">
+    <cfRule type="expression" dxfId="60" priority="55">
       <formula>TRIM(LOWER(AU20))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="52" priority="52" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="59" priority="56" operator="endsWith" text="no">
       <formula>RIGHT(AU20,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW18">
-    <cfRule type="endsWith" dxfId="51" priority="86" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="58" priority="90" operator="endsWith" text="no">
       <formula>RIGHT(AW18,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW18">
-    <cfRule type="expression" dxfId="50" priority="50">
+    <cfRule type="expression" dxfId="57" priority="54">
       <formula>TRIM(LOWER(AW18))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW19">
-    <cfRule type="endsWith" dxfId="49" priority="49" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="56" priority="53" operator="endsWith" text="no">
       <formula>RIGHT(AW19,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW19">
-    <cfRule type="expression" dxfId="48" priority="48">
+    <cfRule type="expression" dxfId="55" priority="52">
       <formula>TRIM(LOWER(AW19))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T9">
-    <cfRule type="expression" dxfId="47" priority="45">
+    <cfRule type="expression" dxfId="54" priority="49">
       <formula>TRIM(LOWER(T9))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="46" priority="46" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="53" priority="50" operator="endsWith" text="no">
       <formula>RIGHT(T9,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI9">
-    <cfRule type="expression" dxfId="45" priority="43">
+    <cfRule type="expression" dxfId="52" priority="47">
       <formula>TRIM(LOWER(AI9))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="44" priority="44" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="51" priority="48" operator="endsWith" text="no">
       <formula>RIGHT(AI9,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T7">
-    <cfRule type="expression" dxfId="43" priority="41">
+    <cfRule type="expression" dxfId="50" priority="45">
       <formula>TRIM(LOWER(T7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="42" priority="42" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="49" priority="46" operator="endsWith" text="no">
       <formula>RIGHT(T7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH7">
-    <cfRule type="expression" dxfId="41" priority="39">
+    <cfRule type="expression" dxfId="48" priority="43">
       <formula>TRIM(LOWER(AH7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="40" priority="40" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="47" priority="44" operator="endsWith" text="no">
       <formula>RIGHT(AH7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:O7">
-    <cfRule type="expression" dxfId="39" priority="37">
+    <cfRule type="expression" dxfId="46" priority="41">
       <formula>TRIM(LOWER(L7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="38" priority="38" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="45" priority="42" operator="endsWith" text="no">
       <formula>RIGHT(L7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O7">
-    <cfRule type="expression" dxfId="37" priority="35">
+    <cfRule type="expression" dxfId="44" priority="39">
       <formula>TRIM(LOWER(O7))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="36" priority="36" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="43" priority="40" operator="endsWith" text="no">
       <formula>RIGHT(O7,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O14">
-    <cfRule type="endsWith" dxfId="35" priority="34" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="42" priority="38" operator="endsWith" text="no">
       <formula>RIGHT(O14,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O14">
-    <cfRule type="expression" dxfId="34" priority="33">
+    <cfRule type="expression" dxfId="41" priority="37">
       <formula>TRIM(LOWER(O14))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O14">
-    <cfRule type="containsBlanks" dxfId="33" priority="32">
+    <cfRule type="containsBlanks" dxfId="40" priority="36">
       <formula>LEN(TRIM(O14))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15">
-    <cfRule type="endsWith" dxfId="32" priority="31" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="39" priority="35" operator="endsWith" text="no">
       <formula>RIGHT(O15,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15">
-    <cfRule type="expression" dxfId="31" priority="30">
+    <cfRule type="expression" dxfId="38" priority="34">
       <formula>TRIM(LOWER(O15))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15">
-    <cfRule type="containsBlanks" dxfId="30" priority="29">
+    <cfRule type="containsBlanks" dxfId="37" priority="33">
       <formula>LEN(TRIM(O15))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF18:BH18">
-    <cfRule type="expression" dxfId="29" priority="27">
+    <cfRule type="expression" dxfId="36" priority="31">
       <formula>TRIM(LOWER(BF18))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="28" priority="28" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="35" priority="32" operator="endsWith" text="no">
       <formula>RIGHT(BF18,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF14:BH14">
-    <cfRule type="expression" dxfId="27" priority="25">
+    <cfRule type="expression" dxfId="34" priority="29">
       <formula>TRIM(LOWER(BF14))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="26" priority="26" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="33" priority="30" operator="endsWith" text="no">
       <formula>RIGHT(BF14,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF12:BH12">
-    <cfRule type="expression" dxfId="25" priority="23">
+    <cfRule type="expression" dxfId="32" priority="27">
       <formula>TRIM(LOWER(BF12))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="24" priority="24" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="31" priority="28" operator="endsWith" text="no">
       <formula>RIGHT(BF12,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF20:BH20">
-    <cfRule type="expression" dxfId="23" priority="21">
+    <cfRule type="expression" dxfId="30" priority="25">
       <formula>TRIM(LOWER(BF20))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="22" priority="22" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="29" priority="26" operator="endsWith" text="no">
       <formula>RIGHT(BF20,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF15:BH15">
-    <cfRule type="expression" dxfId="21" priority="19">
+    <cfRule type="expression" dxfId="28" priority="23">
       <formula>TRIM(LOWER(BF15))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="20" priority="20" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="27" priority="24" operator="endsWith" text="no">
       <formula>RIGHT(BF15,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC13">
-    <cfRule type="endsWith" dxfId="19" priority="18" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="26" priority="22" operator="endsWith" text="no">
       <formula>RIGHT(AC13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC13">
-    <cfRule type="expression" dxfId="18" priority="17">
+    <cfRule type="expression" dxfId="25" priority="21">
       <formula>TRIM(LOWER(AC13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC13">
-    <cfRule type="containsBlanks" dxfId="17" priority="16">
+    <cfRule type="containsBlanks" dxfId="24" priority="20">
       <formula>LEN(TRIM(AC13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD13">
-    <cfRule type="endsWith" dxfId="16" priority="15" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="23" priority="19" operator="endsWith" text="no">
       <formula>RIGHT(AD13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD13">
-    <cfRule type="expression" dxfId="15" priority="14">
+    <cfRule type="expression" dxfId="22" priority="18">
       <formula>TRIM(LOWER(AD13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD13">
-    <cfRule type="containsBlanks" dxfId="14" priority="13">
+    <cfRule type="containsBlanks" dxfId="21" priority="17">
       <formula>LEN(TRIM(AD13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH13">
-    <cfRule type="endsWith" dxfId="13" priority="12" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="20" priority="16" operator="endsWith" text="no">
       <formula>RIGHT(AH13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH13">
-    <cfRule type="expression" dxfId="12" priority="11">
+    <cfRule type="expression" dxfId="19" priority="15">
       <formula>TRIM(LOWER(AH13))&lt;&gt;"no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH13">
-    <cfRule type="containsBlanks" dxfId="11" priority="10">
+    <cfRule type="containsBlanks" dxfId="18" priority="14">
       <formula>LEN(TRIM(AH13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF13:BH13">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="17" priority="12">
       <formula>TRIM(LOWER(BF13))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="9" priority="9" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="16" priority="13" operator="endsWith" text="no">
       <formula>RIGHT(BF13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF13:BH13">
-    <cfRule type="containsBlanks" dxfId="8" priority="7">
+    <cfRule type="containsBlanks" dxfId="15" priority="11">
       <formula>LEN(TRIM(BF13))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BF13:BH13">
-    <cfRule type="expression" dxfId="7" priority="5">
+    <cfRule type="expression" dxfId="14" priority="9">
       <formula>TRIM(LOWER(BF13))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="6" priority="6" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="13" priority="10" operator="endsWith" text="no">
       <formula>RIGHT(BF13,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T9">
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="10" priority="7">
       <formula>TRIM(LOWER(T9))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="2" priority="4" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="9" priority="8" operator="endsWith" text="no">
       <formula>RIGHT(T9,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI9">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>TRIM(LOWER(AI9))&lt;&gt;"no"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="0" priority="2" operator="endsWith" text="no">
+    <cfRule type="endsWith" dxfId="7" priority="6" operator="endsWith" text="no">
       <formula>RIGHT(AI9,LEN("no"))="no"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N10">
+    <cfRule type="expression" dxfId="6" priority="3">
+      <formula>TRIM(LOWER(N10))&lt;&gt;"no"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="5" priority="4" operator="endsWith" text="no">
+      <formula>RIGHT(N10,LEN("no"))="no"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AQ10">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>TRIM(LOWER(AQ10))&lt;&gt;"no"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="3" priority="2" operator="endsWith" text="no">
+      <formula>RIGHT(AQ10,LEN("no"))="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11004,8 +10940,8 @@
     <col min="15" max="15" width="54" style="146" customWidth="1"/>
     <col min="16" max="16" width="41.1640625" style="146" customWidth="1"/>
     <col min="17" max="17" width="5.83203125" style="146" customWidth="1"/>
-    <col min="18" max="18" width="15.83203125" style="146" customWidth="1"/>
-    <col min="19" max="19" width="26.1640625" style="146" customWidth="1"/>
+    <col min="18" max="18" width="20.5" style="146" customWidth="1"/>
+    <col min="19" max="19" width="30.83203125" style="146" customWidth="1"/>
     <col min="20" max="20" width="19.5" style="146" customWidth="1"/>
     <col min="21" max="21" width="43.33203125" style="146" customWidth="1"/>
     <col min="22" max="22" width="5.83203125" style="146" customWidth="1"/>
@@ -11014,15 +10950,15 @@
     <col min="25" max="25" width="19.5" style="146" customWidth="1"/>
     <col min="26" max="26" width="46.5" style="146" customWidth="1"/>
     <col min="27" max="27" width="5.83203125" style="146" customWidth="1"/>
-    <col min="28" max="28" width="16.1640625" style="146" customWidth="1"/>
-    <col min="29" max="29" width="22" style="146" customWidth="1"/>
+    <col min="28" max="28" width="20.83203125" style="146" customWidth="1"/>
+    <col min="29" max="29" width="28.5" style="146" customWidth="1"/>
     <col min="30" max="30" width="20.83203125" style="146" customWidth="1"/>
     <col min="31" max="31" width="41.1640625" style="146" customWidth="1"/>
     <col min="32" max="32" width="5.83203125" style="146" customWidth="1"/>
     <col min="33" max="33" width="23.33203125" style="146" customWidth="1"/>
-    <col min="34" max="34" width="26.1640625" style="146" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="28" style="146" customWidth="1"/>
     <col min="35" max="35" width="42.1640625" style="146" customWidth="1"/>
-    <col min="36" max="36" width="41.6640625" style="146" customWidth="1"/>
+    <col min="36" max="36" width="50" style="146" customWidth="1"/>
     <col min="37" max="37" width="5.83203125" customWidth="1"/>
     <col min="38" max="38" width="24" style="146" customWidth="1"/>
     <col min="39" max="39" width="27" style="146" customWidth="1"/>
@@ -11031,8 +10967,8 @@
     <col min="42" max="42" width="33.33203125" style="146" customWidth="1"/>
     <col min="43" max="43" width="5.83203125" customWidth="1"/>
     <col min="44" max="44" width="45" style="146" customWidth="1"/>
-    <col min="45" max="45" width="49.5" style="146" customWidth="1"/>
-    <col min="46" max="46" width="18.33203125" style="146" customWidth="1"/>
+    <col min="45" max="45" width="57.83203125" style="146" customWidth="1"/>
+    <col min="46" max="46" width="35.1640625" style="146" customWidth="1"/>
     <col min="47" max="16384" width="10.83203125" style="146"/>
   </cols>
   <sheetData>
@@ -11078,7 +11014,7 @@
       <c r="AI6" s="158"/>
       <c r="AJ6" s="158"/>
       <c r="AL6" s="159" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AM6" s="160"/>
       <c r="AN6" s="160"/>
@@ -11094,7 +11030,7 @@
       <c r="C7" s="152"/>
       <c r="D7" s="189"/>
       <c r="E7" s="166" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F7" s="166" t="s">
         <v>261</v>
@@ -11103,7 +11039,7 @@
         <v>262</v>
       </c>
       <c r="H7" s="166" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I7" s="166" t="s">
         <v>263</v>
@@ -11112,7 +11048,7 @@
         <v>264</v>
       </c>
       <c r="K7" s="166" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="L7" s="145"/>
       <c r="M7" s="169" t="s">
@@ -11137,7 +11073,7 @@
       <c r="Z7" s="171"/>
       <c r="AA7" s="147"/>
       <c r="AB7" s="169" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AC7" s="170"/>
       <c r="AD7" s="170"/>
@@ -11150,19 +11086,19 @@
       <c r="AI7" s="170"/>
       <c r="AJ7" s="171"/>
       <c r="AL7" s="172" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="AM7" s="173"/>
       <c r="AN7" s="173"/>
       <c r="AO7" s="174"/>
       <c r="AP7" s="176" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="AR7" s="179" t="s">
         <v>279</v>
       </c>
       <c r="AS7" s="179" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AT7" s="179" t="s">
         <v>280</v>
@@ -11180,67 +11116,67 @@
       <c r="K8" s="165"/>
       <c r="L8" s="145"/>
       <c r="M8" s="181" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N8" s="182"/>
       <c r="O8" s="183"/>
       <c r="P8" s="184" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Q8" s="147"/>
       <c r="R8" s="181" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="S8" s="182"/>
       <c r="T8" s="183"/>
       <c r="U8" s="184" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="V8" s="147"/>
       <c r="W8" s="181" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="X8" s="182"/>
       <c r="Y8" s="183"/>
       <c r="Z8" s="184" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AA8" s="147"/>
       <c r="AB8" s="181" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AC8" s="182"/>
       <c r="AD8" s="183"/>
       <c r="AE8" s="184" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AF8" s="147"/>
       <c r="AG8" s="181" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AH8" s="182"/>
       <c r="AI8" s="183"/>
       <c r="AJ8" s="184" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AL8" s="186" t="s">
+        <v>322</v>
+      </c>
+      <c r="AM8" s="186" t="s">
         <v>323</v>
-      </c>
-      <c r="AM8" s="186" t="s">
-        <v>324</v>
       </c>
       <c r="AN8" s="186" t="s">
         <v>268</v>
       </c>
       <c r="AO8" s="186" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AP8" s="175"/>
       <c r="AR8" s="178"/>
       <c r="AS8" s="178"/>
       <c r="AT8" s="178"/>
     </row>
-    <row r="9" spans="3:61" ht="205" customHeight="1">
+    <row r="9" spans="3:61" ht="199" customHeight="1">
       <c r="C9" s="153"/>
       <c r="D9" s="189"/>
       <c r="E9" s="167"/>
@@ -11360,515 +11296,515 @@
       <c r="AT10" s="189"/>
     </row>
     <row r="11" spans="3:61" ht="195" customHeight="1">
-      <c r="C11" s="191" t="s">
+      <c r="C11" s="193" t="s">
         <v>32</v>
       </c>
       <c r="D11" s="189"/>
-      <c r="E11" s="195" t="str">
+      <c r="E11" s="191" t="str">
         <f>Taxonomy!D7</f>
         <v>✗</v>
       </c>
-      <c r="F11" s="195" t="str">
+      <c r="F11" s="191" t="str">
         <f>Taxonomy!E7</f>
         <v>✗</v>
       </c>
-      <c r="G11" s="195" t="str">
+      <c r="G11" s="191" t="str">
         <f>Taxonomy!F7</f>
         <v>✗</v>
       </c>
-      <c r="H11" s="195" t="str">
+      <c r="H11" s="191" t="str">
         <f>Taxonomy!G7</f>
         <v>✗</v>
       </c>
-      <c r="I11" s="195" t="str">
+      <c r="I11" s="191" t="str">
         <f>Taxonomy!H7</f>
         <v>✗</v>
       </c>
-      <c r="J11" s="195" t="str">
+      <c r="J11" s="191" t="str">
         <f>Taxonomy!I7</f>
         <v>no</v>
       </c>
-      <c r="K11" s="195" t="str">
+      <c r="K11" s="191" t="str">
         <f>Taxonomy!J7</f>
         <v>no</v>
       </c>
       <c r="L11"/>
-      <c r="M11" s="195" t="str">
+      <c r="M11" s="191" t="str">
         <f>Taxonomy!L7</f>
         <v>no</v>
       </c>
-      <c r="N11" s="195" t="str">
+      <c r="N11" s="191" t="str">
         <f>Taxonomy!M7</f>
         <v>no</v>
       </c>
-      <c r="O11" s="195" t="str">
+      <c r="O11" s="191" t="str">
         <f>Taxonomy!N7</f>
         <v>no</v>
       </c>
-      <c r="P11" s="195" t="str">
+      <c r="P11" s="191" t="str">
         <f>Taxonomy!O7</f>
         <v>no</v>
       </c>
       <c r="Q11"/>
-      <c r="R11" s="195" t="str">
+      <c r="R11" s="191" t="str">
         <f>Taxonomy!Q7</f>
         <v>no</v>
       </c>
-      <c r="S11" s="195" t="str">
+      <c r="S11" s="191" t="str">
         <f>Taxonomy!R7</f>
         <v>no</v>
       </c>
-      <c r="T11" s="195" t="str">
+      <c r="T11" s="191" t="str">
         <f>Taxonomy!S7</f>
         <v>no</v>
       </c>
-      <c r="U11" s="195" t="str">
+      <c r="U11" s="191" t="str">
         <f>Taxonomy!T7</f>
         <v>no</v>
       </c>
       <c r="V11"/>
-      <c r="W11" s="195" t="str">
+      <c r="W11" s="191" t="str">
         <f>Taxonomy!V7</f>
         <v>no</v>
       </c>
-      <c r="X11" s="195" t="str">
+      <c r="X11" s="191" t="str">
         <f>Taxonomy!W7</f>
         <v>no</v>
       </c>
-      <c r="Y11" s="195" t="str">
+      <c r="Y11" s="191" t="str">
         <f>Taxonomy!X7</f>
         <v>no</v>
       </c>
-      <c r="Z11" s="195" t="str">
+      <c r="Z11" s="191" t="str">
         <f>Taxonomy!Y7</f>
         <v>no</v>
       </c>
       <c r="AA11"/>
-      <c r="AB11" s="195" t="str">
+      <c r="AB11" s="191" t="str">
         <f>Taxonomy!AA7</f>
         <v>no</v>
       </c>
-      <c r="AC11" s="195" t="str">
+      <c r="AC11" s="191" t="str">
         <f>Taxonomy!AB7</f>
         <v>no</v>
       </c>
-      <c r="AD11" s="195" t="str">
+      <c r="AD11" s="191" t="str">
         <f>Taxonomy!AC7</f>
         <v>no</v>
       </c>
-      <c r="AE11" s="195" t="str">
+      <c r="AE11" s="191" t="str">
         <f>Taxonomy!AD7</f>
         <v>no</v>
       </c>
       <c r="AF11"/>
-      <c r="AG11" s="195" t="str">
+      <c r="AG11" s="191" t="str">
         <f>Taxonomy!AF7</f>
         <v>no</v>
       </c>
-      <c r="AH11" s="195" t="str">
+      <c r="AH11" s="191" t="str">
         <f>Taxonomy!AG7</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="AI11" s="195" t="str">
+      <c r="AI11" s="191" t="str">
         <f>Taxonomy!AH7</f>
-        <v>✗(available for estimations in virtualised
-context )</v>
-      </c>
-      <c r="AJ11" s="195" t="str">
+        <v>no</v>
+      </c>
+      <c r="AJ11" s="191" t="str">
         <f>Taxonomy!AI7</f>
         <v>OS-provided PID CPU %</v>
       </c>
-      <c r="AL11" s="195" t="str">
+      <c r="AL11" s="191" t="str">
         <f>Taxonomy!AK7</f>
         <v>✗</v>
       </c>
-      <c r="AM11" s="195" t="str">
+      <c r="AM11" s="191" t="str">
         <f>Taxonomy!AL7</f>
         <v>no</v>
       </c>
-      <c r="AN11" s="195" t="str">
+      <c r="AN11" s="191" t="str">
         <f>Taxonomy!AM7</f>
         <v>no</v>
       </c>
-      <c r="AO11" s="195" t="str">
+      <c r="AO11" s="191" t="str">
         <f>Taxonomy!AN7</f>
         <v>no</v>
       </c>
-      <c r="AP11" s="195" t="str">
+      <c r="AP11" s="191" t="str">
         <f>Taxonomy!AO7</f>
         <v>no</v>
       </c>
-      <c r="AR11" s="195" t="str">
+      <c r="AR11" s="191" t="str">
         <f>Taxonomy!AQ7</f>
         <v>no</v>
       </c>
-      <c r="AS11" s="195" t="str">
+      <c r="AS11" s="191" t="str">
         <f>Taxonomy!AR7</f>
         <v>✗</v>
       </c>
-      <c r="AT11" s="195" t="str">
+      <c r="AT11" s="191" t="str">
         <f>Taxonomy!AS7</f>
         <v>no</v>
       </c>
     </row>
-    <row r="12" spans="3:61" ht="408" customHeight="1">
-      <c r="C12" s="192" t="s">
-        <v>327</v>
+    <row r="12" spans="3:61" ht="409.5" customHeight="1">
+      <c r="C12" s="194" t="s">
+        <v>326</v>
       </c>
       <c r="D12" s="189"/>
-      <c r="E12" s="195" t="str">
+      <c r="E12" s="191" t="str">
         <f>Taxonomy!D8</f>
         <v>✗</v>
       </c>
-      <c r="F12" s="195" t="str">
+      <c r="F12" s="191" t="str">
         <f>Taxonomy!E8</f>
         <v>✗</v>
       </c>
-      <c r="G12" s="195" t="str">
+      <c r="G12" s="191" t="str">
         <f>Taxonomy!F8</f>
         <v>✗</v>
       </c>
-      <c r="H12" s="195" t="str">
+      <c r="H12" s="191" t="str">
         <f>Taxonomy!G8</f>
         <v>✗</v>
       </c>
-      <c r="I12" s="195" t="str">
+      <c r="I12" s="191" t="str">
         <f>Taxonomy!H8</f>
         <v>✗</v>
       </c>
-      <c r="J12" s="195" t="str">
+      <c r="J12" s="191" t="str">
         <f>Taxonomy!I8</f>
         <v>no</v>
       </c>
-      <c r="K12" s="195" t="str">
+      <c r="K12" s="191" t="str">
         <f>Taxonomy!J8</f>
         <v>no</v>
       </c>
       <c r="L12"/>
-      <c r="M12" s="195" t="str">
+      <c r="M12" s="191" t="str">
         <f>Taxonomy!L8</f>
         <v>no</v>
       </c>
-      <c r="N12" s="195" t="str">
+      <c r="N12" s="191" t="str">
         <f>Taxonomy!M8</f>
         <v>✗ (RAPL)</v>
       </c>
-      <c r="O12" s="195" t="str">
+      <c r="O12" s="191" t="str">
         <f>Taxonomy!N8</f>
         <v>✗Regression-based models for VM deployment</v>
       </c>
-      <c r="P12" s="195" t="str">
+      <c r="P12" s="191" t="str">
         <f>Taxonomy!O8</f>
         <v>OS-provided PID CPU %
 Cgroups Stat</v>
       </c>
       <c r="Q12"/>
-      <c r="R12" s="195" t="str">
+      <c r="R12" s="191" t="str">
         <f>Taxonomy!Q8</f>
         <v>no</v>
       </c>
-      <c r="S12" s="195" t="str">
+      <c r="S12" s="191" t="str">
         <f>Taxonomy!R8</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T12" s="195" t="str">
+      <c r="T12" s="191" t="str">
         <f>Taxonomy!S8</f>
         <v>no</v>
       </c>
-      <c r="U12" s="195" t="str">
+      <c r="U12" s="191" t="str">
         <f>Taxonomy!T8</f>
         <v>OS-provided PID CPU %
 Cgroups Stat</v>
       </c>
       <c r="V12"/>
-      <c r="W12" s="195" t="str">
+      <c r="W12" s="191" t="str">
         <f>Taxonomy!V8</f>
         <v>no</v>
       </c>
-      <c r="X12" s="195" t="str">
+      <c r="X12" s="191" t="str">
         <f>Taxonomy!W8</f>
         <v>✗(NVLM)</v>
       </c>
-      <c r="Y12" s="195" t="str">
+      <c r="Y12" s="191" t="str">
         <f>Taxonomy!X8</f>
         <v>no</v>
       </c>
-      <c r="Z12" s="195" t="str">
+      <c r="Z12" s="191" t="str">
         <f>Taxonomy!Y8</f>
         <v xml:space="preserve">NVLM-provided (i.e. driver) per-process SM utilization </v>
       </c>
       <c r="AA12"/>
-      <c r="AB12" s="195" t="str">
+      <c r="AB12" s="191" t="str">
         <f>Taxonomy!AA8</f>
         <v>no</v>
       </c>
-      <c r="AC12" s="195" t="str">
+      <c r="AC12" s="191" t="str">
         <f>Taxonomy!AB8</f>
         <v>no</v>
       </c>
-      <c r="AD12" s="195" t="str">
+      <c r="AD12" s="191" t="str">
         <f>Taxonomy!AC8</f>
         <v>no</v>
       </c>
-      <c r="AE12" s="195" t="str">
+      <c r="AE12" s="191" t="str">
         <f>Taxonomy!AD8</f>
         <v>no</v>
       </c>
       <c r="AF12"/>
-      <c r="AG12" s="195" t="str">
+      <c r="AG12" s="191" t="str">
         <f>Taxonomy!AF8</f>
         <v>✗(IPMI, ACPI)</v>
       </c>
-      <c r="AH12" s="195" t="str">
+      <c r="AH12" s="191" t="str">
         <f>Taxonomy!AG8</f>
         <v>no</v>
       </c>
-      <c r="AI12" s="195" t="str">
+      <c r="AI12" s="191" t="str">
         <f>Taxonomy!AH8</f>
-        <v>Regression-based 
-trained power model</v>
-      </c>
-      <c r="AJ12" s="195" t="str">
+        <v>Regression-based model</v>
+      </c>
+      <c r="AJ12" s="191" t="str">
         <f>Taxonomy!AI8</f>
         <v>OS-provided PID CPU %
 Cgroups Stat</v>
       </c>
-      <c r="AL12" s="195" t="str">
+      <c r="AL12" s="191" t="str">
         <f>Taxonomy!AK8</f>
         <v>✗</v>
       </c>
-      <c r="AM12" s="195" t="str">
+      <c r="AM12" s="191" t="str">
         <f>Taxonomy!AL8</f>
         <v>no</v>
       </c>
-      <c r="AN12" s="195" t="str">
+      <c r="AN12" s="191" t="str">
         <f>Taxonomy!AM8</f>
         <v>no</v>
       </c>
-      <c r="AO12" s="195" t="str">
+      <c r="AO12" s="191" t="str">
         <f>Taxonomy!AN8</f>
         <v>no</v>
       </c>
-      <c r="AP12" s="195" t="str">
+      <c r="AP12" s="191" t="str">
         <f>Taxonomy!AO8</f>
         <v>Modeled and allocated
 proportionnaly to processes size</v>
       </c>
-      <c r="AR12" s="195" t="str">
+      <c r="AR12" s="191" t="str">
         <f>Taxonomy!AQ8</f>
         <v>Regression model (# CPU and OS-provided Resource Utilisation metrics as input)</v>
       </c>
-      <c r="AS12" s="195" t="str">
+      <c r="AS12" s="191" t="str">
         <f>Taxonomy!AR8</f>
-        <v>( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</v>
-      </c>
-      <c r="AT12" s="195" t="str">
+        <v>no
+( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</v>
+      </c>
+      <c r="AT12" s="191" t="str">
         <f>Taxonomy!AS8</f>
         <v>no</v>
       </c>
     </row>
     <row r="13" spans="3:61" ht="409" customHeight="1">
-      <c r="C13" s="192" t="s">
-        <v>326</v>
+      <c r="C13" s="194" t="s">
+        <v>325</v>
       </c>
       <c r="D13" s="189"/>
-      <c r="E13" s="195" t="str">
+      <c r="E13" s="191" t="str">
         <f>Taxonomy!D9</f>
         <v>✗</v>
       </c>
-      <c r="F13" s="195" t="str">
+      <c r="F13" s="191" t="str">
         <f>Taxonomy!E9</f>
         <v>✗</v>
       </c>
-      <c r="G13" s="195" t="str">
+      <c r="G13" s="191" t="str">
         <f>Taxonomy!F9</f>
         <v>✗</v>
       </c>
-      <c r="H13" s="195" t="str">
+      <c r="H13" s="191" t="str">
         <f>Taxonomy!G9</f>
         <v>✗</v>
       </c>
-      <c r="I13" s="195" t="str">
+      <c r="I13" s="191" t="str">
         <f>Taxonomy!H9</f>
         <v>✗</v>
       </c>
-      <c r="J13" s="195" t="str">
+      <c r="J13" s="191" t="str">
         <f>Taxonomy!I9</f>
         <v>no</v>
       </c>
-      <c r="K13" s="195" t="str">
+      <c r="K13" s="191" t="str">
         <f>Taxonomy!J9</f>
         <v>no</v>
       </c>
       <c r="L13"/>
-      <c r="M13" s="195" t="str">
+      <c r="M13" s="191" t="str">
         <f>Taxonomy!L9</f>
         <v>no</v>
       </c>
-      <c r="N13" s="195" t="str">
+      <c r="N13" s="191" t="str">
         <f>Taxonomy!M9</f>
         <v>✗ (RAPL)</v>
       </c>
-      <c r="O13" s="195" t="str">
+      <c r="O13" s="191" t="str">
         <f>Taxonomy!N9</f>
         <v>✗Regression-based 
  models for VM deployment</v>
       </c>
-      <c r="P13" s="195" t="str">
+      <c r="P13" s="191" t="str">
         <f>Taxonomy!O9</f>
         <v>PID runtime + HPC vector (cycles, instructions, cache misses) through eBPF tracing</v>
       </c>
       <c r="Q13"/>
-      <c r="R13" s="195" t="str">
+      <c r="R13" s="191" t="str">
         <f>Taxonomy!Q9</f>
         <v>no</v>
       </c>
-      <c r="S13" s="195" t="str">
+      <c r="S13" s="191" t="str">
         <f>Taxonomy!R9</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T13" s="195" t="str">
+      <c r="T13" s="191" t="str">
         <f>Taxonomy!S9</f>
         <v>no</v>
       </c>
-      <c r="U13" s="195" t="str">
+      <c r="U13" s="191" t="str">
         <f>Taxonomy!T9</f>
         <v>PID runtime + HPC vector (cycles, instructions, cache misses) through eBPF tracing</v>
       </c>
       <c r="V13"/>
-      <c r="W13" s="195" t="str">
+      <c r="W13" s="191" t="str">
         <f>Taxonomy!V9</f>
         <v>no</v>
       </c>
-      <c r="X13" s="195" t="str">
+      <c r="X13" s="191" t="str">
         <f>Taxonomy!W9</f>
         <v>✗(NVLM)</v>
       </c>
-      <c r="Y13" s="195" t="str">
+      <c r="Y13" s="191" t="str">
         <f>Taxonomy!X9</f>
         <v>no</v>
       </c>
-      <c r="Z13" s="195" t="str">
+      <c r="Z13" s="191" t="str">
         <f>Taxonomy!Y9</f>
         <v xml:space="preserve">NVLM-provided (i.e. driver) per-process SM utilization </v>
       </c>
       <c r="AA13"/>
-      <c r="AB13" s="195" t="str">
+      <c r="AB13" s="191" t="str">
         <f>Taxonomy!AA9</f>
         <v>no</v>
       </c>
-      <c r="AC13" s="195" t="str">
+      <c r="AC13" s="191" t="str">
         <f>Taxonomy!AB9</f>
         <v>no</v>
       </c>
-      <c r="AD13" s="195" t="str">
+      <c r="AD13" s="191" t="str">
         <f>Taxonomy!AC9</f>
         <v>no</v>
       </c>
-      <c r="AE13" s="195" t="str">
+      <c r="AE13" s="191" t="str">
         <f>Taxonomy!AD9</f>
         <v>no</v>
       </c>
       <c r="AF13"/>
-      <c r="AG13" s="195" t="str">
+      <c r="AG13" s="191" t="str">
         <f>Taxonomy!AF9</f>
         <v>✗(IPMI, ACPI)</v>
       </c>
-      <c r="AH13" s="195" t="str">
+      <c r="AH13" s="191" t="str">
         <f>Taxonomy!AG9</f>
         <v>no</v>
       </c>
-      <c r="AI13" s="195" t="str">
+      <c r="AI13" s="191" t="str">
         <f>Taxonomy!AH9</f>
         <v>Regression-based 
 trained power model</v>
       </c>
-      <c r="AJ13" s="195" t="str">
+      <c r="AJ13" s="191" t="str">
         <f>Taxonomy!AI9</f>
         <v>PID runtime + HPC vector (cycles, instructions, cache misses) through eBPF tracing</v>
       </c>
-      <c r="AL13" s="195" t="str">
+      <c r="AL13" s="191" t="str">
         <f>Taxonomy!AK9</f>
         <v>no</v>
       </c>
-      <c r="AM13" s="195" t="str">
+      <c r="AM13" s="191" t="str">
         <f>Taxonomy!AL9</f>
         <v>✗ (from HPC vector  (cycles, instructions, cache misses))</v>
       </c>
-      <c r="AN13" s="195" t="str">
+      <c r="AN13" s="191" t="str">
         <f>Taxonomy!AM9</f>
         <v>no</v>
       </c>
-      <c r="AO13" s="195" t="str">
+      <c r="AO13" s="191" t="str">
         <f>Taxonomy!AN9</f>
         <v>no</v>
       </c>
-      <c r="AP13" s="195" t="str">
+      <c r="AP13" s="191" t="str">
         <f>Taxonomy!AO9</f>
         <v>Modeled and allocated
 proportionnaly to processes size</v>
       </c>
-      <c r="AR13" s="195" t="str">
+      <c r="AR13" s="191" t="str">
         <f>Taxonomy!AQ9</f>
         <v>Regression model (# CPU and OS-provided Resource Utilisation metrics as input)</v>
       </c>
-      <c r="AS13" s="195" t="str">
+      <c r="AS13" s="191" t="str">
         <f>Taxonomy!AR9</f>
-        <v>( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</v>
-      </c>
-      <c r="AT13" s="195" t="str">
+        <v>no
+( (CNCF 2023) mentions a planned "passthrough" mode for VM deployment which expose VM energy in a shared file.</v>
+      </c>
+      <c r="AT13" s="191" t="str">
         <f>Taxonomy!AS9</f>
         <v>no</v>
       </c>
     </row>
-    <row r="14" spans="3:61" ht="362" customHeight="1">
-      <c r="C14" s="193" t="s">
+    <row r="14" spans="3:61" ht="403" customHeight="1">
+      <c r="C14" s="195" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="189"/>
-      <c r="E14" s="195" t="str">
+      <c r="E14" s="191" t="str">
         <f>Taxonomy!D10</f>
         <v>no</v>
       </c>
-      <c r="F14" s="195" t="str">
+      <c r="F14" s="191" t="str">
         <f>Taxonomy!E10</f>
         <v>no</v>
       </c>
-      <c r="G14" s="195" t="str">
+      <c r="G14" s="191" t="str">
         <f>Taxonomy!F10</f>
         <v>✗</v>
       </c>
-      <c r="H14" s="195" t="str">
+      <c r="H14" s="191" t="str">
         <f>Taxonomy!G10</f>
         <v>no</v>
       </c>
-      <c r="I14" s="195" t="str">
+      <c r="I14" s="191" t="str">
         <f>Taxonomy!H10</f>
         <v>no</v>
       </c>
-      <c r="J14" s="195" t="str">
+      <c r="J14" s="191" t="str">
         <f>Taxonomy!I10</f>
         <v>no</v>
       </c>
-      <c r="K14" s="195" t="str">
+      <c r="K14" s="191" t="str">
         <f>Taxonomy!J10</f>
         <v>✗(SCI functionnality)</v>
       </c>
       <c r="L14"/>
-      <c r="M14" s="195" t="str">
+      <c r="M14" s="191" t="str">
         <f>Taxonomy!L10</f>
         <v>✗(Compatible with certain Metric Providers)</v>
       </c>
-      <c r="N14" s="195" t="str">
+      <c r="N14" s="191" t="str">
         <f>Taxonomy!M10</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="O14" s="195" t="str">
+      <c r="O14" s="191" t="str">
         <f>Taxonomy!N10</f>
-        <v>✗XGBoost (TDP)
-or Regression-based (TDP)</v>
-      </c>
-      <c r="P14" s="195" t="str">
+        <v xml:space="preserve">✗1) XGBoost model (TDP, Machine Specs and CPU%)
+2) Analytical Model(TDP, #CPUchips and CPU %) </v>
+      </c>
+      <c r="P14" s="191" t="str">
         <f>Taxonomy!O10</f>
         <v xml:space="preserve">OS-provided PID CPU %
 Cgroups Stat
@@ -11876,19 +11812,19 @@
 </v>
       </c>
       <c r="Q14"/>
-      <c r="R14" s="195" t="str">
+      <c r="R14" s="191" t="str">
         <f>Taxonomy!Q10</f>
         <v>no</v>
       </c>
-      <c r="S14" s="195" t="str">
+      <c r="S14" s="191" t="str">
         <f>Taxonomy!R10</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T14" s="195" t="str">
+      <c r="T14" s="191" t="str">
         <f>Taxonomy!S10</f>
         <v>no</v>
       </c>
-      <c r="U14" s="195" t="str">
+      <c r="U14" s="191" t="str">
         <f>Taxonomy!T10</f>
         <v xml:space="preserve">OS-provided PID CPU %
 Cgroups Stat (Container)
@@ -11896,19 +11832,19 @@
 </v>
       </c>
       <c r="V14"/>
-      <c r="W14" s="195" t="str">
+      <c r="W14" s="191" t="str">
         <f>Taxonomy!V10</f>
         <v>no</v>
       </c>
-      <c r="X14" s="195" t="str">
+      <c r="X14" s="191" t="str">
         <f>Taxonomy!W10</f>
         <v>✗(NVLM)</v>
       </c>
-      <c r="Y14" s="195" t="str">
+      <c r="Y14" s="191" t="str">
         <f>Taxonomy!X10</f>
         <v>no</v>
       </c>
-      <c r="Z14" s="195" t="str">
+      <c r="Z14" s="191" t="str">
         <f>Taxonomy!Y10</f>
         <v xml:space="preserve">OS-provided PID CPU %
 Cgroups Stat
@@ -11916,74 +11852,74 @@
 </v>
       </c>
       <c r="AA14"/>
-      <c r="AB14" s="195" t="str">
+      <c r="AB14" s="191" t="str">
         <f>Taxonomy!AA10</f>
         <v>no</v>
       </c>
-      <c r="AC14" s="195" t="str">
+      <c r="AC14" s="191" t="str">
         <f>Taxonomy!AB10</f>
         <v>no</v>
       </c>
-      <c r="AD14" s="195" t="str">
+      <c r="AD14" s="191" t="str">
         <f>Taxonomy!AC10</f>
         <v>no</v>
       </c>
-      <c r="AE14" s="195" t="str">
+      <c r="AE14" s="191" t="str">
         <f>Taxonomy!AD10</f>
         <v>no</v>
       </c>
       <c r="AF14"/>
-      <c r="AG14" s="195" t="str">
+      <c r="AG14" s="191" t="str">
         <f>Taxonomy!AF10</f>
         <v>✗</v>
       </c>
-      <c r="AH14" s="195" t="str">
+      <c r="AH14" s="191" t="str">
         <f>Taxonomy!AG10</f>
         <v>✗(RAPL PSYS Domain)</v>
       </c>
-      <c r="AI14" s="195" t="str">
+      <c r="AI14" s="191" t="str">
         <f>Taxonomy!AH10</f>
-        <v xml:space="preserve">✗XGBoost model for system-level estimations in virtualised
-contex (TDP) </v>
-      </c>
-      <c r="AJ14" s="195" t="str">
+        <v xml:space="preserve">✗1) XGBoost model (TDP, Machine Specs and CPU%)
+2) Analytical Model(TDP, #CPUchips and CPU %) </v>
+      </c>
+      <c r="AJ14" s="191" t="str">
         <f>Taxonomy!AI10</f>
         <v>OS-provided PID CPU %
 Cgroups Stat (container)
 Code Special Print (Code Section)</v>
       </c>
-      <c r="AL14" s="195" t="str">
+      <c r="AL14" s="191" t="str">
         <f>Taxonomy!AK10</f>
         <v>✗</v>
       </c>
-      <c r="AM14" s="195" t="str">
+      <c r="AM14" s="191" t="str">
         <f>Taxonomy!AL10</f>
         <v>no</v>
       </c>
-      <c r="AN14" s="195" t="str">
+      <c r="AN14" s="191" t="str">
         <f>Taxonomy!AM10</f>
         <v>no</v>
       </c>
-      <c r="AO14" s="195" t="str">
+      <c r="AO14" s="191" t="str">
         <f>Taxonomy!AN10</f>
         <v>✗(SCI functionnality)</v>
       </c>
-      <c r="AP14" s="195" t="str">
+      <c r="AP14" s="191" t="str">
         <f>Taxonomy!AO10</f>
         <v>Modeled and 
 allocated to container 
 according to OS-provided PID CPU %</v>
       </c>
-      <c r="AR14" s="195" t="str">
+      <c r="AR14" s="191" t="str">
         <f>Taxonomy!AQ10</f>
-        <v xml:space="preserve">XGBoost Model (#CPU TDP, CPU Frequency and CPU % as input)
-</v>
-      </c>
-      <c r="AS14" s="195" t="str">
+        <v xml:space="preserve">1) XGBoost model (TDP, Machine Specs and CPU%)
+2) Analytical Model(TDP, #CPUchips and CPU %) </v>
+      </c>
+      <c r="AS14" s="191" t="str">
         <f>Taxonomy!AR10</f>
         <v>no</v>
       </c>
-      <c r="AT14" s="195" t="str">
+      <c r="AT14" s="191" t="str">
         <f>Taxonomy!AS10</f>
         <v>no</v>
       </c>
@@ -11992,647 +11928,647 @@
       <c r="C15" s="145"/>
       <c r="D15" s="189"/>
       <c r="E15"/>
-      <c r="F15" s="196"/>
-      <c r="G15" s="196"/>
-      <c r="H15" s="196"/>
-      <c r="I15" s="196"/>
-      <c r="J15" s="196"/>
-      <c r="K15" s="196"/>
+      <c r="F15" s="192"/>
+      <c r="G15" s="192"/>
+      <c r="H15" s="192"/>
+      <c r="I15" s="192"/>
+      <c r="J15" s="192"/>
+      <c r="K15" s="192"/>
       <c r="L15"/>
-      <c r="M15" s="196"/>
-      <c r="N15" s="196"/>
-      <c r="O15" s="196"/>
-      <c r="P15" s="196"/>
+      <c r="M15" s="192"/>
+      <c r="N15" s="192"/>
+      <c r="O15" s="192"/>
+      <c r="P15" s="192"/>
       <c r="Q15"/>
-      <c r="R15" s="196"/>
-      <c r="S15" s="196"/>
-      <c r="T15" s="196"/>
-      <c r="U15" s="196"/>
+      <c r="R15" s="192"/>
+      <c r="S15" s="192"/>
+      <c r="T15" s="192"/>
+      <c r="U15" s="192"/>
       <c r="V15"/>
-      <c r="W15" s="196"/>
-      <c r="X15" s="196"/>
-      <c r="Y15" s="196"/>
-      <c r="Z15" s="196"/>
+      <c r="W15" s="192"/>
+      <c r="X15" s="192"/>
+      <c r="Y15" s="192"/>
+      <c r="Z15" s="192"/>
       <c r="AA15"/>
-      <c r="AB15" s="196"/>
-      <c r="AC15" s="196"/>
-      <c r="AD15" s="196"/>
-      <c r="AE15" s="196"/>
+      <c r="AB15" s="192"/>
+      <c r="AC15" s="192"/>
+      <c r="AD15" s="192"/>
+      <c r="AE15" s="192"/>
       <c r="AF15"/>
-      <c r="AG15" s="196"/>
-      <c r="AH15" s="196"/>
-      <c r="AI15" s="196"/>
-      <c r="AJ15" s="196"/>
-      <c r="AL15" s="196"/>
-      <c r="AM15" s="196"/>
-      <c r="AN15" s="196"/>
-      <c r="AO15" s="196"/>
-      <c r="AP15" s="196"/>
-      <c r="AR15" s="196"/>
-      <c r="AS15" s="196"/>
-      <c r="AT15" s="196"/>
-    </row>
-    <row r="16" spans="3:61" ht="248" customHeight="1">
-      <c r="C16" s="191" t="s">
+      <c r="AG15" s="192"/>
+      <c r="AH15" s="192"/>
+      <c r="AI15" s="192"/>
+      <c r="AJ15" s="192"/>
+      <c r="AL15" s="192"/>
+      <c r="AM15" s="192"/>
+      <c r="AN15" s="192"/>
+      <c r="AO15" s="192"/>
+      <c r="AP15" s="192"/>
+      <c r="AR15" s="192"/>
+      <c r="AS15" s="192"/>
+      <c r="AT15" s="192"/>
+    </row>
+    <row r="16" spans="3:61" ht="320" customHeight="1">
+      <c r="C16" s="193" t="s">
         <v>266</v>
       </c>
       <c r="D16" s="189"/>
-      <c r="E16" s="195" t="str">
+      <c r="E16" s="191" t="str">
         <f>Taxonomy!D12</f>
         <v>no</v>
       </c>
-      <c r="F16" s="195" t="str">
+      <c r="F16" s="191" t="str">
         <f>Taxonomy!E12</f>
         <v>no</v>
       </c>
-      <c r="G16" s="195" t="str">
+      <c r="G16" s="191" t="str">
         <f>Taxonomy!F12</f>
         <v>no</v>
       </c>
-      <c r="H16" s="195" t="str">
+      <c r="H16" s="191" t="str">
         <f>Taxonomy!G12</f>
         <v>no</v>
       </c>
-      <c r="I16" s="195" t="str">
+      <c r="I16" s="191" t="str">
         <f>Taxonomy!H12</f>
         <v>✗</v>
       </c>
-      <c r="J16" s="195" t="str">
+      <c r="J16" s="191" t="str">
         <f>Taxonomy!I12</f>
         <v>no</v>
       </c>
-      <c r="K16" s="195" t="str">
+      <c r="K16" s="191" t="str">
         <f>Taxonomy!J12</f>
         <v>no</v>
       </c>
       <c r="L16"/>
-      <c r="M16" s="195" t="str">
+      <c r="M16" s="191" t="str">
         <f>Taxonomy!L12</f>
         <v>no</v>
       </c>
-      <c r="N16" s="195" t="str">
+      <c r="N16" s="191" t="str">
         <f>Taxonomy!M12</f>
         <v>no</v>
       </c>
-      <c r="O16" s="195" t="str">
+      <c r="O16" s="191" t="str">
         <f>Taxonomy!N12</f>
         <v xml:space="preserve">✗ Linear Regression Model (HPC : "instructions", "cache references", "cache misses" </v>
       </c>
-      <c r="P16" s="195" t="str">
+      <c r="P16" s="191" t="str">
         <f>Taxonomy!O12</f>
         <v>OS-provided PID CPU %</v>
       </c>
       <c r="Q16"/>
-      <c r="R16" s="195" t="str">
+      <c r="R16" s="191" t="str">
         <f>Taxonomy!Q12</f>
         <v>no</v>
       </c>
-      <c r="S16" s="195" t="str">
+      <c r="S16" s="191" t="str">
         <f>Taxonomy!R12</f>
         <v>no</v>
       </c>
-      <c r="T16" s="195" t="str">
+      <c r="T16" s="191" t="str">
         <f>Taxonomy!S12</f>
         <v>no</v>
       </c>
-      <c r="U16" s="195" t="str">
+      <c r="U16" s="191" t="str">
         <f>Taxonomy!T12</f>
         <v>no</v>
       </c>
       <c r="V16"/>
-      <c r="W16" s="195" t="str">
+      <c r="W16" s="191" t="str">
         <f>Taxonomy!V12</f>
         <v>no</v>
       </c>
-      <c r="X16" s="195" t="str">
+      <c r="X16" s="191" t="str">
         <f>Taxonomy!W12</f>
         <v>no</v>
       </c>
-      <c r="Y16" s="195" t="str">
+      <c r="Y16" s="191" t="str">
         <f>Taxonomy!X12</f>
         <v>no</v>
       </c>
-      <c r="Z16" s="195" t="str">
+      <c r="Z16" s="191" t="str">
         <f>Taxonomy!Y12</f>
         <v>no</v>
       </c>
       <c r="AA16"/>
-      <c r="AB16" s="195" t="str">
+      <c r="AB16" s="191" t="str">
         <f>Taxonomy!AA12</f>
         <v>no</v>
       </c>
-      <c r="AC16" s="195" t="str">
+      <c r="AC16" s="191" t="str">
         <f>Taxonomy!AB12</f>
         <v>no</v>
       </c>
-      <c r="AD16" s="195" t="str">
+      <c r="AD16" s="191" t="str">
         <f>Taxonomy!AC12</f>
         <v>✗</v>
       </c>
-      <c r="AE16" s="195" t="str">
+      <c r="AE16" s="191" t="str">
         <f>Taxonomy!AD12</f>
         <v>OS provided per-process (PID)Network I/O</v>
       </c>
       <c r="AF16"/>
-      <c r="AG16" s="195" t="str">
+      <c r="AG16" s="191" t="str">
         <f>Taxonomy!AF12</f>
         <v>no</v>
       </c>
-      <c r="AH16" s="195" t="str">
+      <c r="AH16" s="191" t="str">
         <f>Taxonomy!AG12</f>
         <v>no</v>
       </c>
-      <c r="AI16" s="195" t="str">
+      <c r="AI16" s="191" t="str">
         <f>Taxonomy!AH12</f>
         <v>✗(TDP)</v>
       </c>
-      <c r="AJ16" s="195" t="str">
+      <c r="AJ16" s="191" t="str">
         <f>Taxonomy!AI12</f>
         <v>OS-provided PID CPU %</v>
       </c>
-      <c r="AL16" s="195" t="str">
+      <c r="AL16" s="191" t="str">
         <f>Taxonomy!AK12</f>
         <v>✗</v>
       </c>
-      <c r="AM16" s="195" t="str">
+      <c r="AM16" s="191" t="str">
         <f>Taxonomy!AL12</f>
         <v>no</v>
       </c>
-      <c r="AN16" s="195" t="str">
+      <c r="AN16" s="191" t="str">
         <f>Taxonomy!AM12</f>
         <v>no</v>
       </c>
-      <c r="AO16" s="195" t="str">
+      <c r="AO16" s="191" t="str">
         <f>Taxonomy!AN12</f>
         <v>no</v>
       </c>
-      <c r="AP16" s="195" t="str">
+      <c r="AP16" s="191" t="str">
         <f>Taxonomy!AO12</f>
         <v>no</v>
       </c>
-      <c r="AR16" s="195" t="str">
+      <c r="AR16" s="191" t="str">
         <f>Taxonomy!AQ12</f>
         <v>no</v>
       </c>
-      <c r="AS16" s="195" t="str">
+      <c r="AS16" s="191" t="str">
         <f>Taxonomy!AR12</f>
         <v>no</v>
       </c>
-      <c r="AT16" s="195" t="str">
+      <c r="AT16" s="191" t="str">
         <f>Taxonomy!AS12</f>
         <v>no</v>
       </c>
     </row>
     <row r="17" spans="3:46" ht="263" customHeight="1">
-      <c r="C17" s="193" t="s">
+      <c r="C17" s="195" t="s">
         <v>44</v>
       </c>
       <c r="D17" s="189"/>
-      <c r="E17" s="195" t="str">
+      <c r="E17" s="191" t="str">
         <f>Taxonomy!D13</f>
         <v>no</v>
       </c>
-      <c r="F17" s="195" t="str">
+      <c r="F17" s="191" t="str">
         <f>Taxonomy!E13</f>
         <v>no</v>
       </c>
-      <c r="G17" s="195" t="str">
+      <c r="G17" s="191" t="str">
         <f>Taxonomy!F13</f>
         <v>no</v>
       </c>
-      <c r="H17" s="195" t="str">
+      <c r="H17" s="191" t="str">
         <f>Taxonomy!G13</f>
         <v>no</v>
       </c>
-      <c r="I17" s="195" t="str">
+      <c r="I17" s="191" t="str">
         <f>Taxonomy!H13</f>
         <v>✗</v>
       </c>
-      <c r="J17" s="195" t="str">
+      <c r="J17" s="191" t="str">
         <f>Taxonomy!I13</f>
         <v>no</v>
       </c>
-      <c r="K17" s="195" t="str">
+      <c r="K17" s="191" t="str">
         <f>Taxonomy!J13</f>
         <v>no</v>
       </c>
       <c r="L17"/>
-      <c r="M17" s="195" t="str">
+      <c r="M17" s="191" t="str">
         <f>Taxonomy!L13</f>
         <v>no</v>
       </c>
-      <c r="N17" s="195" t="str">
+      <c r="N17" s="191" t="str">
         <f>Taxonomy!M13</f>
         <v>no</v>
       </c>
-      <c r="O17" s="195" t="str">
+      <c r="O17" s="191" t="str">
         <f>Taxonomy!N13</f>
         <v>✗HPC vector (cycles, instructions, cache misses)</v>
       </c>
-      <c r="P17" s="195" t="str">
+      <c r="P17" s="191" t="str">
         <f>Taxonomy!O13</f>
         <v>OS-provided PID CPU %</v>
       </c>
       <c r="Q17"/>
-      <c r="R17" s="195" t="str">
+      <c r="R17" s="191" t="str">
         <f>Taxonomy!Q13</f>
         <v>no</v>
       </c>
-      <c r="S17" s="195" t="str">
+      <c r="S17" s="191" t="str">
         <f>Taxonomy!R13</f>
         <v>no</v>
       </c>
-      <c r="T17" s="195" t="str">
+      <c r="T17" s="191" t="str">
         <f>Taxonomy!S13</f>
         <v>no</v>
       </c>
-      <c r="U17" s="195" t="str">
+      <c r="U17" s="191" t="str">
         <f>Taxonomy!T13</f>
         <v>no</v>
       </c>
       <c r="V17"/>
-      <c r="W17" s="195" t="str">
+      <c r="W17" s="191" t="str">
         <f>Taxonomy!V13</f>
         <v>no</v>
       </c>
-      <c r="X17" s="195" t="str">
+      <c r="X17" s="191" t="str">
         <f>Taxonomy!W13</f>
         <v>no</v>
       </c>
-      <c r="Y17" s="195" t="str">
+      <c r="Y17" s="191" t="str">
         <f>Taxonomy!X13</f>
         <v>no</v>
       </c>
-      <c r="Z17" s="195" t="str">
+      <c r="Z17" s="191" t="str">
         <f>Taxonomy!Y13</f>
         <v>no</v>
       </c>
       <c r="AA17"/>
-      <c r="AB17" s="195" t="str">
+      <c r="AB17" s="191" t="str">
         <f>Taxonomy!AA13</f>
         <v>no</v>
       </c>
-      <c r="AC17" s="195" t="str">
+      <c r="AC17" s="191" t="str">
         <f>Taxonomy!AB13</f>
         <v>no</v>
       </c>
-      <c r="AD17" s="195" t="str">
+      <c r="AD17" s="191" t="str">
         <f>Taxonomy!AC13</f>
         <v>no</v>
       </c>
-      <c r="AE17" s="195" t="str">
+      <c r="AE17" s="191" t="str">
         <f>Taxonomy!AD13</f>
         <v>no</v>
       </c>
       <c r="AF17"/>
-      <c r="AG17" s="195" t="str">
+      <c r="AG17" s="191" t="str">
         <f>Taxonomy!AF13</f>
         <v>no</v>
       </c>
-      <c r="AH17" s="195" t="str">
+      <c r="AH17" s="191" t="str">
         <f>Taxonomy!AG13</f>
         <v>no</v>
       </c>
-      <c r="AI17" s="195" t="str">
+      <c r="AI17" s="191" t="str">
         <f>Taxonomy!AH13</f>
         <v>✗  HPC     (cycles, instructions, cache misses) vector</v>
       </c>
-      <c r="AJ17" s="195" t="str">
+      <c r="AJ17" s="191" t="str">
         <f>Taxonomy!AI13</f>
         <v>OS-provided PID CPU %</v>
       </c>
-      <c r="AL17" s="195" t="str">
+      <c r="AL17" s="191" t="str">
         <f>Taxonomy!AK13</f>
         <v>✗</v>
       </c>
-      <c r="AM17" s="195" t="str">
+      <c r="AM17" s="191" t="str">
         <f>Taxonomy!AL13</f>
         <v>no</v>
       </c>
-      <c r="AN17" s="195" t="str">
+      <c r="AN17" s="191" t="str">
         <f>Taxonomy!AM13</f>
         <v>no</v>
       </c>
-      <c r="AO17" s="195" t="str">
+      <c r="AO17" s="191" t="str">
         <f>Taxonomy!AN13</f>
         <v>no</v>
       </c>
-      <c r="AP17" s="195" t="str">
+      <c r="AP17" s="191" t="str">
         <f>Taxonomy!AO13</f>
         <v>no</v>
       </c>
-      <c r="AR17" s="195" t="str">
+      <c r="AR17" s="191" t="str">
         <f>Taxonomy!AQ13</f>
         <v>no</v>
       </c>
-      <c r="AS17" s="195" t="str">
+      <c r="AS17" s="191" t="str">
         <f>Taxonomy!AR13</f>
         <v>no</v>
       </c>
-      <c r="AT17" s="195" t="str">
+      <c r="AT17" s="191" t="str">
         <f>Taxonomy!AS13</f>
         <v>no</v>
       </c>
     </row>
     <row r="18" spans="3:46" ht="269" customHeight="1">
-      <c r="C18" s="193" t="s">
+      <c r="C18" s="195" t="s">
         <v>48</v>
       </c>
       <c r="D18" s="189"/>
-      <c r="E18" s="195" t="str">
+      <c r="E18" s="191" t="str">
         <f>Taxonomy!D14</f>
         <v>✗</v>
       </c>
-      <c r="F18" s="195" t="str">
+      <c r="F18" s="191" t="str">
         <f>Taxonomy!E14</f>
         <v>no</v>
       </c>
-      <c r="G18" s="195" t="str">
+      <c r="G18" s="191" t="str">
         <f>Taxonomy!F14</f>
         <v>no</v>
       </c>
-      <c r="H18" s="195" t="str">
+      <c r="H18" s="191" t="str">
         <f>Taxonomy!G14</f>
         <v>✗</v>
       </c>
-      <c r="I18" s="195" t="str">
+      <c r="I18" s="191" t="str">
         <f>Taxonomy!H14</f>
         <v>✗</v>
       </c>
-      <c r="J18" s="195" t="str">
+      <c r="J18" s="191" t="str">
         <f>Taxonomy!I14</f>
         <v>no</v>
       </c>
-      <c r="K18" s="195" t="str">
+      <c r="K18" s="191" t="str">
         <f>Taxonomy!J14</f>
         <v>no</v>
       </c>
       <c r="L18"/>
-      <c r="M18" s="195" t="str">
+      <c r="M18" s="191" t="str">
         <f>Taxonomy!L14</f>
         <v>no</v>
       </c>
-      <c r="N18" s="195" t="str">
+      <c r="N18" s="191" t="str">
         <f>Taxonomy!M14</f>
         <v>✗ (RAPL throush powercap)</v>
       </c>
-      <c r="O18" s="195" t="str">
+      <c r="O18" s="191" t="str">
         <f>Taxonomy!N14</f>
         <v>no</v>
       </c>
-      <c r="P18" s="195" t="str">
+      <c r="P18" s="191" t="str">
         <f>Taxonomy!O14</f>
         <v>OS-provided PID CPU %</v>
       </c>
       <c r="Q18"/>
-      <c r="R18" s="195" t="str">
+      <c r="R18" s="191" t="str">
         <f>Taxonomy!Q14</f>
         <v>no</v>
       </c>
-      <c r="S18" s="195" t="str">
+      <c r="S18" s="191" t="str">
         <f>Taxonomy!R14</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T18" s="195" t="str">
+      <c r="T18" s="191" t="str">
         <f>Taxonomy!S14</f>
         <v>no</v>
       </c>
-      <c r="U18" s="195" t="str">
+      <c r="U18" s="191" t="str">
         <f>Taxonomy!T14</f>
         <v>PID CPU %</v>
       </c>
       <c r="V18"/>
-      <c r="W18" s="195" t="str">
+      <c r="W18" s="191" t="str">
         <f>Taxonomy!V14</f>
         <v>no</v>
       </c>
-      <c r="X18" s="195" t="str">
+      <c r="X18" s="191" t="str">
         <f>Taxonomy!W14</f>
         <v>✗(NVIDIA-SMI, AMD-SMI) (computers and servers)</v>
       </c>
-      <c r="Y18" s="195" t="str">
+      <c r="Y18" s="191" t="str">
         <f>Taxonomy!X14</f>
         <v>no</v>
       </c>
-      <c r="Z18" s="195" t="str">
+      <c r="Z18" s="191" t="str">
         <f>Taxonomy!Y14</f>
         <v>PID GPU % (from driver API)</v>
       </c>
       <c r="AA18"/>
-      <c r="AB18" s="195" t="str">
+      <c r="AB18" s="191" t="str">
         <f>Taxonomy!AA14</f>
         <v>no</v>
       </c>
-      <c r="AC18" s="195" t="str">
+      <c r="AC18" s="191" t="str">
         <f>Taxonomy!AB14</f>
         <v>no</v>
       </c>
-      <c r="AD18" s="195" t="str">
+      <c r="AD18" s="191" t="str">
         <f>Taxonomy!AC14</f>
         <v>no</v>
       </c>
-      <c r="AE18" s="195" t="str">
+      <c r="AE18" s="191" t="str">
         <f>Taxonomy!AD14</f>
         <v>no</v>
       </c>
       <c r="AF18"/>
-      <c r="AG18" s="195" t="str">
+      <c r="AG18" s="191" t="str">
         <f>Taxonomy!AF14</f>
         <v>no</v>
       </c>
-      <c r="AH18" s="195" t="str">
+      <c r="AH18" s="191" t="str">
         <f>Taxonomy!AG14</f>
         <v>no</v>
       </c>
-      <c r="AI18" s="195" t="str">
+      <c r="AI18" s="191" t="str">
         <f>Taxonomy!AH14</f>
         <v>polynomial regression For Rasberry Pi</v>
       </c>
-      <c r="AJ18" s="195" t="str">
+      <c r="AJ18" s="191" t="str">
         <f>Taxonomy!AI14</f>
         <v>OS-provided PID CPU %</v>
       </c>
-      <c r="AL18" s="195" t="str">
+      <c r="AL18" s="191" t="str">
         <f>Taxonomy!AK14</f>
         <v>✗</v>
       </c>
-      <c r="AM18" s="195" t="str">
+      <c r="AM18" s="191" t="str">
         <f>Taxonomy!AL14</f>
         <v>no</v>
       </c>
-      <c r="AN18" s="195" t="str">
+      <c r="AN18" s="191" t="str">
         <f>Taxonomy!AM14</f>
         <v>no</v>
       </c>
-      <c r="AO18" s="195" t="str">
+      <c r="AO18" s="191" t="str">
         <f>Taxonomy!AN14</f>
         <v>no</v>
       </c>
-      <c r="AP18" s="195" t="str">
+      <c r="AP18" s="191" t="str">
         <f>Taxonomy!AO14</f>
         <v>no</v>
       </c>
-      <c r="AR18" s="195" t="str">
+      <c r="AR18" s="191" t="str">
         <f>Taxonomy!AQ14</f>
         <v>no</v>
       </c>
-      <c r="AS18" s="195" t="str">
+      <c r="AS18" s="191" t="str">
         <f>Taxonomy!AR14</f>
         <v>✗</v>
       </c>
-      <c r="AT18" s="195" t="str">
+      <c r="AT18" s="191" t="str">
         <f>Taxonomy!AS14</f>
         <v>no</v>
       </c>
     </row>
     <row r="19" spans="3:46" ht="350" customHeight="1">
-      <c r="C19" s="193" t="s">
+      <c r="C19" s="195" t="s">
         <v>215</v>
       </c>
       <c r="D19" s="189"/>
-      <c r="E19" s="195" t="str">
+      <c r="E19" s="191" t="str">
         <f>Taxonomy!D15</f>
         <v>✗</v>
       </c>
-      <c r="F19" s="195" t="str">
+      <c r="F19" s="191" t="str">
         <f>Taxonomy!E15</f>
         <v>no</v>
       </c>
-      <c r="G19" s="195" t="str">
+      <c r="G19" s="191" t="str">
         <f>Taxonomy!F15</f>
         <v>no</v>
       </c>
-      <c r="H19" s="195" t="str">
+      <c r="H19" s="191" t="str">
         <f>Taxonomy!G15</f>
         <v>✗</v>
       </c>
-      <c r="I19" s="195" t="str">
+      <c r="I19" s="191" t="str">
         <f>Taxonomy!H15</f>
         <v>✗</v>
       </c>
-      <c r="J19" s="195" t="str">
+      <c r="J19" s="191" t="str">
         <f>Taxonomy!I15</f>
         <v>no</v>
       </c>
-      <c r="K19" s="195" t="str">
+      <c r="K19" s="191" t="str">
         <f>Taxonomy!J15</f>
         <v>no</v>
       </c>
       <c r="L19"/>
-      <c r="M19" s="195" t="str">
+      <c r="M19" s="191" t="str">
         <f>Taxonomy!L15</f>
         <v>no</v>
       </c>
-      <c r="N19" s="195" t="str">
+      <c r="N19" s="191" t="str">
         <f>Taxonomy!M15</f>
         <v>✗ (RAPL (linux/windows) or powerMetrics (Mac))</v>
       </c>
-      <c r="O19" s="195" t="str">
+      <c r="O19" s="191" t="str">
         <f>Taxonomy!N15</f>
         <v>no</v>
       </c>
-      <c r="P19" s="195" t="str">
+      <c r="P19" s="191" t="str">
         <f>Taxonomy!O15</f>
         <v>OS-provided PID CPU %</v>
       </c>
       <c r="Q19"/>
-      <c r="R19" s="195" t="str">
+      <c r="R19" s="191" t="str">
         <f>Taxonomy!Q15</f>
         <v>no</v>
       </c>
-      <c r="S19" s="195" t="str">
+      <c r="S19" s="191" t="str">
         <f>Taxonomy!R15</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T19" s="195" t="str">
+      <c r="T19" s="191" t="str">
         <f>Taxonomy!S15</f>
         <v>no</v>
       </c>
-      <c r="U19" s="195" t="str">
+      <c r="U19" s="191" t="str">
         <f>Taxonomy!T15</f>
         <v>PID CPU %</v>
       </c>
       <c r="V19"/>
-      <c r="W19" s="195" t="str">
+      <c r="W19" s="191" t="str">
         <f>Taxonomy!V15</f>
         <v>no</v>
       </c>
-      <c r="X19" s="195" t="str">
+      <c r="X19" s="191" t="str">
         <f>Taxonomy!W15</f>
         <v>✗(NVIDIA-SMI, AMD-SMI) (computers and servers)</v>
       </c>
-      <c r="Y19" s="195" t="str">
+      <c r="Y19" s="191" t="str">
         <f>Taxonomy!X15</f>
         <v>no</v>
       </c>
-      <c r="Z19" s="195" t="str">
+      <c r="Z19" s="191" t="str">
         <f>Taxonomy!Y15</f>
         <v>PID GPU % (from driver API)</v>
       </c>
       <c r="AA19"/>
-      <c r="AB19" s="195" t="str">
+      <c r="AB19" s="191" t="str">
         <f>Taxonomy!AA15</f>
         <v>no</v>
       </c>
-      <c r="AC19" s="195" t="str">
+      <c r="AC19" s="191" t="str">
         <f>Taxonomy!AB15</f>
         <v>no</v>
       </c>
-      <c r="AD19" s="195" t="str">
+      <c r="AD19" s="191" t="str">
         <f>Taxonomy!AC15</f>
         <v>no</v>
       </c>
-      <c r="AE19" s="195" t="str">
+      <c r="AE19" s="191" t="str">
         <f>Taxonomy!AD15</f>
         <v>no</v>
       </c>
       <c r="AF19"/>
-      <c r="AG19" s="195" t="str">
+      <c r="AG19" s="191" t="str">
         <f>Taxonomy!AF15</f>
         <v>no</v>
       </c>
-      <c r="AH19" s="195" t="str">
+      <c r="AH19" s="191" t="str">
         <f>Taxonomy!AG15</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="AI19" s="195" t="str">
+      <c r="AI19" s="191" t="str">
         <f>Taxonomy!AH15</f>
         <v>polynomial regression For Rasberry Pi</v>
       </c>
-      <c r="AJ19" s="195" t="str">
+      <c r="AJ19" s="191" t="str">
         <f>Taxonomy!AI15</f>
         <v>OS-provided PID CPU %</v>
       </c>
-      <c r="AL19" s="195" t="str">
+      <c r="AL19" s="191" t="str">
         <f>Taxonomy!AK15</f>
         <v>✗</v>
       </c>
-      <c r="AM19" s="195" t="str">
+      <c r="AM19" s="191" t="str">
         <f>Taxonomy!AL15</f>
         <v>no</v>
       </c>
-      <c r="AN19" s="195" t="str">
+      <c r="AN19" s="191" t="str">
         <f>Taxonomy!AM15</f>
         <v>no</v>
       </c>
-      <c r="AO19" s="195" t="str">
+      <c r="AO19" s="191" t="str">
         <f>Taxonomy!AN15</f>
         <v>no</v>
       </c>
-      <c r="AP19" s="195" t="str">
+      <c r="AP19" s="191" t="str">
         <f>Taxonomy!AO15</f>
         <v>Modeled and 
 substracted before allocation</v>
       </c>
-      <c r="AR19" s="195" t="str">
+      <c r="AR19" s="191" t="str">
         <f>Taxonomy!AQ15</f>
         <v>no</v>
       </c>
-      <c r="AS19" s="195" t="str">
+      <c r="AS19" s="191" t="str">
         <f>Taxonomy!AR15</f>
         <v>✗</v>
       </c>
-      <c r="AT19" s="195" t="str">
+      <c r="AT19" s="191" t="str">
         <f>Taxonomy!AS15</f>
         <v>no</v>
       </c>
@@ -12641,652 +12577,652 @@
       <c r="C20" s="145"/>
       <c r="D20" s="189"/>
       <c r="E20"/>
-      <c r="F20" s="196"/>
-      <c r="G20" s="196"/>
-      <c r="H20" s="196"/>
-      <c r="I20" s="196"/>
-      <c r="J20" s="196"/>
-      <c r="K20" s="196"/>
+      <c r="F20" s="192"/>
+      <c r="G20" s="192"/>
+      <c r="H20" s="192"/>
+      <c r="I20" s="192"/>
+      <c r="J20" s="192"/>
+      <c r="K20" s="192"/>
       <c r="L20"/>
-      <c r="M20" s="196"/>
-      <c r="N20" s="196"/>
-      <c r="O20" s="196"/>
-      <c r="P20" s="196"/>
+      <c r="M20" s="192"/>
+      <c r="N20" s="192"/>
+      <c r="O20" s="192"/>
+      <c r="P20" s="192"/>
       <c r="Q20"/>
-      <c r="R20" s="196"/>
-      <c r="S20" s="196"/>
-      <c r="T20" s="196"/>
-      <c r="U20" s="196"/>
+      <c r="R20" s="192"/>
+      <c r="S20" s="192"/>
+      <c r="T20" s="192"/>
+      <c r="U20" s="192"/>
       <c r="V20"/>
-      <c r="W20" s="196"/>
-      <c r="X20" s="196"/>
-      <c r="Y20" s="196"/>
-      <c r="Z20" s="196"/>
+      <c r="W20" s="192"/>
+      <c r="X20" s="192"/>
+      <c r="Y20" s="192"/>
+      <c r="Z20" s="192"/>
       <c r="AA20"/>
-      <c r="AB20" s="196"/>
-      <c r="AC20" s="196"/>
-      <c r="AD20" s="196"/>
-      <c r="AE20" s="196"/>
+      <c r="AB20" s="192"/>
+      <c r="AC20" s="192"/>
+      <c r="AD20" s="192"/>
+      <c r="AE20" s="192"/>
       <c r="AF20"/>
-      <c r="AG20" s="196"/>
-      <c r="AH20" s="196"/>
-      <c r="AI20" s="196"/>
-      <c r="AJ20" s="196"/>
-      <c r="AL20" s="196"/>
-      <c r="AM20" s="196"/>
-      <c r="AN20" s="196"/>
-      <c r="AO20" s="196"/>
-      <c r="AP20" s="196"/>
-      <c r="AR20" s="196"/>
-      <c r="AS20" s="196"/>
-      <c r="AT20" s="196"/>
-    </row>
-    <row r="21" spans="3:46" ht="322" customHeight="1">
-      <c r="C21" s="194" t="s">
+      <c r="AG20" s="192"/>
+      <c r="AH20" s="192"/>
+      <c r="AI20" s="192"/>
+      <c r="AJ20" s="192"/>
+      <c r="AL20" s="192"/>
+      <c r="AM20" s="192"/>
+      <c r="AN20" s="192"/>
+      <c r="AO20" s="192"/>
+      <c r="AP20" s="192"/>
+      <c r="AR20" s="192"/>
+      <c r="AS20" s="192"/>
+      <c r="AT20" s="192"/>
+    </row>
+    <row r="21" spans="3:46" ht="354" customHeight="1">
+      <c r="C21" s="196" t="s">
         <v>267</v>
       </c>
       <c r="D21" s="189"/>
-      <c r="E21" s="195" t="str">
+      <c r="E21" s="191" t="str">
         <f>Taxonomy!D17</f>
         <v>no</v>
       </c>
-      <c r="F21" s="195" t="str">
+      <c r="F21" s="191" t="str">
         <f>Taxonomy!E17</f>
         <v>no</v>
       </c>
-      <c r="G21" s="195" t="str">
+      <c r="G21" s="191" t="str">
         <f>Taxonomy!F17</f>
         <v>no</v>
       </c>
-      <c r="H21" s="195" t="str">
+      <c r="H21" s="191" t="str">
         <f>Taxonomy!G17</f>
         <v>no</v>
       </c>
-      <c r="I21" s="195" t="str">
+      <c r="I21" s="191" t="str">
         <f>Taxonomy!H17</f>
         <v>no</v>
       </c>
-      <c r="J21" s="195" t="str">
+      <c r="J21" s="191" t="str">
         <f>Taxonomy!I17</f>
         <v>✗</v>
       </c>
-      <c r="K21" s="195" t="str">
+      <c r="K21" s="191" t="str">
         <f>Taxonomy!J17</f>
         <v>✗</v>
       </c>
       <c r="L21"/>
-      <c r="M21" s="195" t="str">
+      <c r="M21" s="191" t="str">
         <f>Taxonomy!L17</f>
         <v>no</v>
       </c>
-      <c r="N21" s="195" t="str">
+      <c r="N21" s="191" t="str">
         <f>Taxonomy!M17</f>
         <v>no</v>
       </c>
-      <c r="O21" s="195" t="str">
+      <c r="O21" s="191" t="str">
         <f>Taxonomy!N17</f>
         <v>✗ (TDP) Through PowerAPI</v>
       </c>
-      <c r="P21" s="195" t="str">
+      <c r="P21" s="191" t="str">
         <f>Taxonomy!O17</f>
         <v>1) Time Markers : JVM byte code  instrumentation /
 2) Call stack</v>
       </c>
       <c r="Q21"/>
-      <c r="R21" s="195" t="str">
+      <c r="R21" s="191" t="str">
         <f>Taxonomy!Q17</f>
         <v>no</v>
       </c>
-      <c r="S21" s="195" t="str">
+      <c r="S21" s="191" t="str">
         <f>Taxonomy!R17</f>
         <v>no</v>
       </c>
-      <c r="T21" s="195" t="str">
+      <c r="T21" s="191" t="str">
         <f>Taxonomy!S17</f>
         <v>no</v>
       </c>
-      <c r="U21" s="195" t="str">
+      <c r="U21" s="191" t="str">
         <f>Taxonomy!T17</f>
         <v>no</v>
       </c>
       <c r="V21"/>
-      <c r="W21" s="195" t="str">
+      <c r="W21" s="191" t="str">
         <f>Taxonomy!V17</f>
         <v>no</v>
       </c>
-      <c r="X21" s="195" t="str">
+      <c r="X21" s="191" t="str">
         <f>Taxonomy!W17</f>
         <v>no</v>
       </c>
-      <c r="Y21" s="195" t="str">
+      <c r="Y21" s="191" t="str">
         <f>Taxonomy!X17</f>
         <v>no</v>
       </c>
-      <c r="Z21" s="195" t="str">
+      <c r="Z21" s="191" t="str">
         <f>Taxonomy!Y17</f>
         <v>no</v>
       </c>
       <c r="AA21"/>
-      <c r="AB21" s="195" t="str">
+      <c r="AB21" s="191" t="str">
         <f>Taxonomy!AA17</f>
         <v>no</v>
       </c>
-      <c r="AC21" s="195" t="str">
+      <c r="AC21" s="191" t="str">
         <f>Taxonomy!AB17</f>
         <v>no</v>
       </c>
-      <c r="AD21" s="195" t="str">
+      <c r="AD21" s="191" t="str">
         <f>Taxonomy!AC17</f>
         <v>✗(Through PowerAPI)</v>
       </c>
-      <c r="AE21" s="195" t="str">
+      <c r="AE21" s="191" t="str">
         <f>Taxonomy!AD17</f>
         <v xml:space="preserve"> getInputStream()  getOutputStream() calls</v>
       </c>
       <c r="AF21"/>
-      <c r="AG21" s="195" t="str">
+      <c r="AG21" s="191" t="str">
         <f>Taxonomy!AF17</f>
         <v>no</v>
       </c>
-      <c r="AH21" s="195" t="str">
+      <c r="AH21" s="191" t="str">
         <f>Taxonomy!AG17</f>
         <v>no</v>
       </c>
-      <c r="AI21" s="195" t="str">
+      <c r="AI21" s="191" t="str">
         <f>Taxonomy!AH17</f>
         <v>no</v>
       </c>
-      <c r="AJ21" s="195" t="str">
+      <c r="AJ21" s="191" t="str">
         <f>Taxonomy!AI17</f>
         <v>no</v>
       </c>
-      <c r="AL21" s="195" t="str">
+      <c r="AL21" s="191" t="str">
         <f>Taxonomy!AK17</f>
         <v>✗ (For NIC)</v>
       </c>
-      <c r="AM21" s="195" t="str">
+      <c r="AM21" s="191" t="str">
         <f>Taxonomy!AL17</f>
         <v>no</v>
       </c>
-      <c r="AN21" s="195" t="str">
+      <c r="AN21" s="191" t="str">
         <f>Taxonomy!AM17</f>
         <v>✗(for CPU : call-stack sampling version)</v>
       </c>
-      <c r="AO21" s="195" t="str">
+      <c r="AO21" s="191" t="str">
         <f>Taxonomy!AN17</f>
         <v>✗ (for CPU : bytecode instrumentation version)</v>
       </c>
-      <c r="AP21" s="195" t="str">
+      <c r="AP21" s="191" t="str">
         <f>Taxonomy!AO17</f>
         <v>no</v>
       </c>
-      <c r="AR21" s="195" t="str">
+      <c r="AR21" s="191" t="str">
         <f>Taxonomy!AQ17</f>
         <v>no</v>
       </c>
-      <c r="AS21" s="195" t="str">
+      <c r="AS21" s="191" t="str">
         <f>Taxonomy!AR17</f>
         <v>no</v>
       </c>
-      <c r="AT21" s="195" t="str">
+      <c r="AT21" s="191" t="str">
         <f>Taxonomy!AS17</f>
         <v>no</v>
       </c>
     </row>
     <row r="22" spans="3:46" ht="409.5" customHeight="1">
-      <c r="C22" s="192" t="s">
+      <c r="C22" s="194" t="s">
         <v>223</v>
       </c>
       <c r="D22" s="189"/>
-      <c r="E22" s="195" t="str">
+      <c r="E22" s="191" t="str">
         <f>Taxonomy!D18</f>
         <v>no</v>
       </c>
-      <c r="F22" s="195" t="str">
+      <c r="F22" s="191" t="str">
         <f>Taxonomy!E18</f>
         <v>no</v>
       </c>
-      <c r="G22" s="195" t="str">
+      <c r="G22" s="191" t="str">
         <f>Taxonomy!F18</f>
         <v>no</v>
       </c>
-      <c r="H22" s="195" t="str">
+      <c r="H22" s="191" t="str">
         <f>Taxonomy!G18</f>
         <v>no</v>
       </c>
-      <c r="I22" s="195" t="str">
+      <c r="I22" s="191" t="str">
         <f>Taxonomy!H18</f>
         <v>no</v>
       </c>
-      <c r="J22" s="195" t="str">
+      <c r="J22" s="191" t="str">
         <f>Taxonomy!I18</f>
         <v>✗</v>
       </c>
-      <c r="K22" s="195" t="str">
+      <c r="K22" s="191" t="str">
         <f>Taxonomy!J18</f>
         <v>✗</v>
       </c>
       <c r="L22"/>
-      <c r="M22" s="195" t="str">
+      <c r="M22" s="191" t="str">
         <f>Taxonomy!L18</f>
         <v>no</v>
       </c>
-      <c r="N22" s="195" t="str">
+      <c r="N22" s="191" t="str">
         <f>Taxonomy!M18</f>
         <v>✗ (RAPL through powercap)</v>
       </c>
-      <c r="O22" s="195" t="str">
+      <c r="O22" s="191" t="str">
         <f>Taxonomy!N18</f>
         <v>no</v>
       </c>
-      <c r="P22" s="195" t="str">
+      <c r="P22" s="191" t="str">
         <f>Taxonomy!O18</f>
         <v>1) OS-provided PID CPU %  for Java Threads through JVM instrumentation
 2) Call Stack</v>
       </c>
       <c r="Q22"/>
-      <c r="R22" s="195" t="str">
+      <c r="R22" s="191" t="str">
         <f>Taxonomy!Q18</f>
         <v>no</v>
       </c>
-      <c r="S22" s="195" t="str">
+      <c r="S22" s="191" t="str">
         <f>Taxonomy!R18</f>
         <v>✗(RAPL) Through Power Joular</v>
       </c>
-      <c r="T22" s="195" t="str">
+      <c r="T22" s="191" t="str">
         <f>Taxonomy!S18</f>
         <v>no</v>
       </c>
-      <c r="U22" s="195" t="str">
+      <c r="U22" s="191" t="str">
         <f>Taxonomy!T18</f>
         <v>1) OS-provided PID CPU % for Java Threads through JVM instrumentation
 2) Statistical sampling of thread stack trace</v>
       </c>
       <c r="V22"/>
-      <c r="W22" s="195" t="str">
+      <c r="W22" s="191" t="str">
         <f>Taxonomy!V18</f>
         <v>no</v>
       </c>
-      <c r="X22" s="195" t="str">
+      <c r="X22" s="191" t="str">
         <f>Taxonomy!W18</f>
         <v>✗(NVIDIA SMI) (computers and servers through Power Joular</v>
       </c>
-      <c r="Y22" s="195" t="str">
+      <c r="Y22" s="191" t="str">
         <f>Taxonomy!X18</f>
         <v>no</v>
       </c>
-      <c r="Z22" s="195" t="str">
+      <c r="Z22" s="191" t="str">
         <f>Taxonomy!Y18</f>
         <v>1) OS-provided PID CPU % for Java Threads through JVM instrumentation
 2) Statistical sampling of thread stack trace</v>
       </c>
       <c r="AA22"/>
-      <c r="AB22" s="195" t="str">
+      <c r="AB22" s="191" t="str">
         <f>Taxonomy!AA18</f>
         <v>no</v>
       </c>
-      <c r="AC22" s="195" t="str">
+      <c r="AC22" s="191" t="str">
         <f>Taxonomy!AB18</f>
         <v>no</v>
       </c>
-      <c r="AD22" s="195" t="str">
+      <c r="AD22" s="191" t="str">
         <f>Taxonomy!AC18</f>
         <v>no</v>
       </c>
-      <c r="AE22" s="195" t="str">
+      <c r="AE22" s="191" t="str">
         <f>Taxonomy!AD18</f>
         <v>no</v>
       </c>
       <c r="AF22"/>
-      <c r="AG22" s="195" t="str">
+      <c r="AG22" s="191" t="str">
         <f>Taxonomy!AF18</f>
         <v>no</v>
       </c>
-      <c r="AH22" s="195" t="str">
+      <c r="AH22" s="191" t="str">
         <f>Taxonomy!AG18</f>
         <v>no</v>
       </c>
-      <c r="AI22" s="195" t="str">
+      <c r="AI22" s="191" t="str">
         <f>Taxonomy!AH18</f>
         <v>polynomial regression For Rasberry Pi</v>
       </c>
-      <c r="AJ22" s="195" t="str">
+      <c r="AJ22" s="191" t="str">
         <f>Taxonomy!AI18</f>
         <v>1) OS-provided PID CPU % for Java Threads through JVM instrumentation
 2) Statistical sampling of thread stack trace</v>
       </c>
-      <c r="AL22" s="195" t="str">
+      <c r="AL22" s="191" t="str">
         <f>Taxonomy!AK18</f>
         <v>✗(for threads)</v>
       </c>
-      <c r="AM22" s="195" t="str">
+      <c r="AM22" s="191" t="str">
         <f>Taxonomy!AL18</f>
         <v>no</v>
       </c>
-      <c r="AN22" s="195" t="str">
+      <c r="AN22" s="191" t="str">
         <f>Taxonomy!AM18</f>
         <v>✗</v>
       </c>
-      <c r="AO22" s="195" t="str">
+      <c r="AO22" s="191" t="str">
         <f>Taxonomy!AN18</f>
         <v>no</v>
       </c>
-      <c r="AP22" s="195" t="str">
+      <c r="AP22" s="191" t="str">
         <f>Taxonomy!AO18</f>
         <v>no</v>
       </c>
-      <c r="AR22" s="195" t="str">
+      <c r="AR22" s="191" t="str">
         <f>Taxonomy!AQ18</f>
         <v>no</v>
       </c>
-      <c r="AS22" s="195" t="str">
+      <c r="AS22" s="191" t="str">
         <f>Taxonomy!AR18</f>
         <v>no</v>
       </c>
-      <c r="AT22" s="195" t="str">
+      <c r="AT22" s="191" t="str">
         <f>Taxonomy!AS18</f>
         <v>Uses PowerJoular</v>
       </c>
     </row>
     <row r="23" spans="3:46" ht="409" customHeight="1">
-      <c r="C23" s="192" t="s">
+      <c r="C23" s="194" t="s">
         <v>196</v>
       </c>
       <c r="D23" s="189"/>
-      <c r="E23" s="195" t="str">
+      <c r="E23" s="191" t="str">
         <f>Taxonomy!D19</f>
         <v>✗</v>
       </c>
-      <c r="F23" s="195" t="str">
+      <c r="F23" s="191" t="str">
         <f>Taxonomy!E19</f>
         <v>no</v>
       </c>
-      <c r="G23" s="195" t="str">
+      <c r="G23" s="191" t="str">
         <f>Taxonomy!F19</f>
         <v>no</v>
       </c>
-      <c r="H23" s="195" t="str">
+      <c r="H23" s="191" t="str">
         <f>Taxonomy!G19</f>
         <v>✗</v>
       </c>
-      <c r="I23" s="195" t="str">
+      <c r="I23" s="191" t="str">
         <f>Taxonomy!H19</f>
         <v>✗</v>
       </c>
-      <c r="J23" s="195" t="str">
+      <c r="J23" s="191" t="str">
         <f>Taxonomy!I19</f>
         <v>✗</v>
       </c>
-      <c r="K23" s="195" t="str">
+      <c r="K23" s="191" t="str">
         <f>Taxonomy!J19</f>
         <v>✗</v>
       </c>
       <c r="L23"/>
-      <c r="M23" s="195" t="str">
+      <c r="M23" s="191" t="str">
         <f>Taxonomy!L19</f>
         <v>no</v>
       </c>
-      <c r="N23" s="195" t="str">
+      <c r="N23" s="191" t="str">
         <f>Taxonomy!M19</f>
         <v>✗ (RAPL throush PAPI)</v>
       </c>
-      <c r="O23" s="195" t="str">
+      <c r="O23" s="191" t="str">
         <f>Taxonomy!N19</f>
         <v>no</v>
       </c>
-      <c r="P23" s="195" t="str">
+      <c r="P23" s="191" t="str">
         <f>Taxonomy!O19</f>
         <v>Call stack</v>
       </c>
       <c r="Q23"/>
-      <c r="R23" s="195" t="str">
+      <c r="R23" s="191" t="str">
         <f>Taxonomy!Q19</f>
         <v>no</v>
       </c>
-      <c r="S23" s="195" t="str">
+      <c r="S23" s="191" t="str">
         <f>Taxonomy!R19</f>
         <v>✗(RAPL)</v>
       </c>
-      <c r="T23" s="195" t="str">
+      <c r="T23" s="191" t="str">
         <f>Taxonomy!S19</f>
         <v>no</v>
       </c>
-      <c r="U23" s="195" t="str">
+      <c r="U23" s="191" t="str">
         <f>Taxonomy!T19</f>
         <v>Call stack sampling</v>
       </c>
       <c r="V23"/>
-      <c r="W23" s="195" t="str">
+      <c r="W23" s="191" t="str">
         <f>Taxonomy!V19</f>
         <v>no</v>
       </c>
-      <c r="X23" s="195" t="str">
+      <c r="X23" s="191" t="str">
         <f>Taxonomy!W19</f>
         <v>no</v>
       </c>
-      <c r="Y23" s="195" t="str">
+      <c r="Y23" s="191" t="str">
         <f>Taxonomy!X19</f>
         <v>no</v>
       </c>
-      <c r="Z23" s="195" t="str">
+      <c r="Z23" s="191" t="str">
         <f>Taxonomy!Y19</f>
         <v>no</v>
       </c>
       <c r="AA23"/>
-      <c r="AB23" s="195" t="str">
+      <c r="AB23" s="191" t="str">
         <f>Taxonomy!AA19</f>
         <v>no</v>
       </c>
-      <c r="AC23" s="195" t="str">
+      <c r="AC23" s="191" t="str">
         <f>Taxonomy!AB19</f>
         <v>no</v>
       </c>
-      <c r="AD23" s="195" t="str">
+      <c r="AD23" s="191" t="str">
         <f>Taxonomy!AC19</f>
         <v>no</v>
       </c>
-      <c r="AE23" s="195" t="str">
+      <c r="AE23" s="191" t="str">
         <f>Taxonomy!AD19</f>
         <v>no</v>
       </c>
       <c r="AF23"/>
-      <c r="AG23" s="195" t="str">
+      <c r="AG23" s="191" t="str">
         <f>Taxonomy!AF19</f>
         <v>no</v>
       </c>
-      <c r="AH23" s="195" t="str">
+      <c r="AH23" s="191" t="str">
         <f>Taxonomy!AG19</f>
         <v>✗ (RAPL throush PAPI)</v>
       </c>
-      <c r="AI23" s="195" t="str">
+      <c r="AI23" s="191" t="str">
         <f>Taxonomy!AH19</f>
         <v>no</v>
       </c>
-      <c r="AJ23" s="195" t="str">
+      <c r="AJ23" s="191" t="str">
         <f>Taxonomy!AI19</f>
         <v>Call stack sampling</v>
       </c>
-      <c r="AL23" s="195" t="str">
+      <c r="AL23" s="191" t="str">
         <f>Taxonomy!AK19</f>
         <v>no</v>
       </c>
-      <c r="AM23" s="195" t="str">
+      <c r="AM23" s="191" t="str">
         <f>Taxonomy!AL19</f>
         <v>no</v>
       </c>
-      <c r="AN23" s="195" t="str">
+      <c r="AN23" s="191" t="str">
         <f>Taxonomy!AM19</f>
         <v>✗(1) Allocate all RAPL system energy to process it is attached to
 2) Statistical Sampling (stack trace) to allocate energy to functions)</v>
       </c>
-      <c r="AO23" s="195" t="str">
+      <c r="AO23" s="191" t="str">
         <f>Taxonomy!AN19</f>
         <v>no</v>
       </c>
-      <c r="AP23" s="195" t="str">
+      <c r="AP23" s="191" t="str">
         <f>Taxonomy!AO19</f>
         <v>no</v>
       </c>
-      <c r="AR23" s="195" t="str">
+      <c r="AR23" s="191" t="str">
         <f>Taxonomy!AQ19</f>
         <v>no</v>
       </c>
-      <c r="AS23" s="195" t="str">
+      <c r="AS23" s="191" t="str">
         <f>Taxonomy!AR19</f>
         <v>no</v>
       </c>
-      <c r="AT23" s="195" t="str">
+      <c r="AT23" s="191" t="str">
         <f>Taxonomy!AS19</f>
         <v>no</v>
       </c>
     </row>
-    <row r="24" spans="3:46" ht="283" customHeight="1">
-      <c r="C24" s="192" t="s">
+    <row r="24" spans="3:46" ht="377" customHeight="1">
+      <c r="C24" s="194" t="s">
         <v>42</v>
       </c>
       <c r="D24" s="189"/>
-      <c r="E24" s="195" t="str">
+      <c r="E24" s="191" t="str">
         <f>Taxonomy!D20</f>
         <v>no</v>
       </c>
-      <c r="F24" s="195" t="str">
+      <c r="F24" s="191" t="str">
         <f>Taxonomy!E20</f>
         <v>no</v>
       </c>
-      <c r="G24" s="195" t="str">
+      <c r="G24" s="191" t="str">
         <f>Taxonomy!F20</f>
         <v>no</v>
       </c>
-      <c r="H24" s="195" t="str">
+      <c r="H24" s="191" t="str">
         <f>Taxonomy!G20</f>
         <v>no</v>
       </c>
-      <c r="I24" s="195" t="str">
+      <c r="I24" s="191" t="str">
         <f>Taxonomy!H20</f>
         <v>no</v>
       </c>
-      <c r="J24" s="195" t="str">
+      <c r="J24" s="191" t="str">
         <f>Taxonomy!I20</f>
         <v>no</v>
       </c>
-      <c r="K24" s="195" t="str">
+      <c r="K24" s="191" t="str">
         <f>Taxonomy!J20</f>
         <v>✗</v>
       </c>
       <c r="L24"/>
-      <c r="M24" s="195" t="str">
+      <c r="M24" s="191" t="str">
         <f>Taxonomy!L20</f>
         <v>no</v>
       </c>
-      <c r="N24" s="195" t="str">
+      <c r="N24" s="191" t="str">
         <f>Taxonomy!M20</f>
         <v>✗ (RAPL through linux  MSR kernel module)</v>
       </c>
-      <c r="O24" s="195" t="str">
+      <c r="O24" s="191" t="str">
         <f>Taxonomy!N20</f>
         <v>no</v>
       </c>
-      <c r="P24" s="195" t="str">
+      <c r="P24" s="191" t="str">
         <f>Taxonomy!O20</f>
         <v>Time Markers</v>
       </c>
       <c r="Q24"/>
-      <c r="R24" s="195" t="str">
+      <c r="R24" s="191" t="str">
         <f>Taxonomy!Q20</f>
         <v>no</v>
       </c>
-      <c r="S24" s="195" t="str">
+      <c r="S24" s="191" t="str">
         <f>Taxonomy!R20</f>
         <v>✗ (RAPL through linux  MSR kernel module)</v>
       </c>
-      <c r="T24" s="195" t="str">
+      <c r="T24" s="191" t="str">
         <f>Taxonomy!S20</f>
         <v>no</v>
       </c>
-      <c r="U24" s="195" t="str">
+      <c r="U24" s="191" t="str">
         <f>Taxonomy!T20</f>
         <v>Time Markers</v>
       </c>
       <c r="V24"/>
-      <c r="W24" s="195" t="str">
+      <c r="W24" s="191" t="str">
         <f>Taxonomy!V20</f>
         <v>no</v>
       </c>
-      <c r="X24" s="195" t="str">
+      <c r="X24" s="191" t="str">
         <f>Taxonomy!W20</f>
         <v>no</v>
       </c>
-      <c r="Y24" s="195" t="str">
+      <c r="Y24" s="191" t="str">
         <f>Taxonomy!X20</f>
         <v>no</v>
       </c>
-      <c r="Z24" s="195" t="str">
+      <c r="Z24" s="191" t="str">
         <f>Taxonomy!Y20</f>
         <v>no</v>
       </c>
       <c r="AA24"/>
-      <c r="AB24" s="195" t="str">
+      <c r="AB24" s="191" t="str">
         <f>Taxonomy!AA20</f>
         <v>no</v>
       </c>
-      <c r="AC24" s="195" t="str">
+      <c r="AC24" s="191" t="str">
         <f>Taxonomy!AB20</f>
         <v>no</v>
       </c>
-      <c r="AD24" s="195" t="str">
+      <c r="AD24" s="191" t="str">
         <f>Taxonomy!AC20</f>
         <v>no</v>
       </c>
-      <c r="AE24" s="195" t="str">
+      <c r="AE24" s="191" t="str">
         <f>Taxonomy!AD20</f>
         <v>no</v>
       </c>
       <c r="AF24"/>
-      <c r="AG24" s="195" t="str">
+      <c r="AG24" s="191" t="str">
         <f>Taxonomy!AF20</f>
         <v>no</v>
       </c>
-      <c r="AH24" s="195" t="str">
+      <c r="AH24" s="191" t="str">
         <f>Taxonomy!AG20</f>
         <v>✗ (RAPL through linux  MSR kernel module)</v>
       </c>
-      <c r="AI24" s="195" t="str">
+      <c r="AI24" s="191" t="str">
         <f>Taxonomy!AH20</f>
         <v>no</v>
       </c>
-      <c r="AJ24" s="195" t="str">
+      <c r="AJ24" s="191" t="str">
         <f>Taxonomy!AI20</f>
         <v>Time Markers</v>
       </c>
-      <c r="AL24" s="195" t="str">
+      <c r="AL24" s="191" t="str">
         <f>Taxonomy!AK20</f>
         <v>no</v>
       </c>
-      <c r="AM24" s="195" t="str">
+      <c r="AM24" s="191" t="str">
         <f>Taxonomy!AL20</f>
         <v>no</v>
       </c>
-      <c r="AN24" s="195" t="str">
+      <c r="AN24" s="191" t="str">
         <f>Taxonomy!AM20</f>
         <v>no</v>
       </c>
-      <c r="AO24" s="195" t="str">
+      <c r="AO24" s="191" t="str">
         <f>Taxonomy!AN20</f>
         <v>✗</v>
       </c>
-      <c r="AP24" s="195" t="str">
+      <c r="AP24" s="191" t="str">
         <f>Taxonomy!AO20</f>
         <v>no</v>
       </c>
-      <c r="AR24" s="195" t="str">
+      <c r="AR24" s="191" t="str">
         <f>Taxonomy!AQ20</f>
         <v>no</v>
       </c>
-      <c r="AS24" s="195" t="str">
+      <c r="AS24" s="191" t="str">
         <f>Taxonomy!AR20</f>
         <v>no</v>
       </c>
-      <c r="AT24" s="195" t="str">
+      <c r="AT24" s="191" t="str">
         <f>Taxonomy!AS20</f>
         <v>no</v>
       </c>
@@ -13332,10 +13268,10 @@
     <mergeCell ref="H7:H9"/>
   </mergeCells>
   <conditionalFormatting sqref="E11:K14 AL11:AP24 AR11:AT24 M11:P24 R11:U24 W11:Z24 AB11:AE24 AG11:AJ24 E21:K24 F20:K20 E16:K19 F15:K15">
-    <cfRule type="beginsWith" dxfId="5" priority="1" stopIfTrue="1" operator="beginsWith" text="no">
+    <cfRule type="beginsWith" dxfId="12" priority="1" stopIfTrue="1" operator="beginsWith" text="no">
       <formula>LEFT(E11,LEN("no"))="no"</formula>
     </cfRule>
-    <cfRule type="notContainsBlanks" dxfId="4" priority="7" stopIfTrue="1">
+    <cfRule type="notContainsBlanks" dxfId="11" priority="7" stopIfTrue="1">
       <formula>LEN(TRIM(E11))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>